<commit_message>
Add employee photo box beside the personal-info table
- Upload in the form (JPG/PNG/WebP, max 15 MB) with live preview and remove
- Normalized in memory: EXIF rotation applied, metadata stripped, resized,
  never stretched (contain-fit) in the form, report view, print and Excel
- Template: photo box B6:D19; personal info moved to E-M, personnel N-X
- Markdown embeds the photo; shared workbooks with pictures stay appendable
- Pillow added as a dependency

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Template/report_template.xlsx
+++ b/Template/report_template.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +38,11 @@
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="B Nazanin"/>
+      <color rgb="009A9AB0"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="B Nazanin"/>
@@ -226,7 +231,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -235,90 +240,93 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" indent="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" indent="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1" indent="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
@@ -785,14 +793,14 @@
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>اطلاعات پرسنلی</t>
-        </is>
-      </c>
+      <c r="K4" s="2" t="n"/>
       <c r="L4" s="2" t="n"/>
       <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="n"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>اطلاعات پرسنلی</t>
+        </is>
+      </c>
       <c r="O4" s="2" t="n"/>
       <c r="P4" s="2" t="n"/>
       <c r="Q4" s="2" t="n"/>
@@ -832,47 +840,51 @@
     <row r="6" ht="30" customHeight="1">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>نام ونام خانوادگی</t>
+          <t>عکس کارمند</t>
         </is>
       </c>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="3" t="n"/>
-      <c r="E6" s="4" t="n"/>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>نام ونام خانوادگی</t>
+        </is>
+      </c>
       <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="4" t="n"/>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="5" t="n"/>
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>متأهل</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="M6" s="6" t="inlineStr">
         <is>
           <t>مجرد</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>نوع استخدام</t>
         </is>
       </c>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="5" t="n"/>
-      <c r="N6" s="4" t="n"/>
-      <c r="O6" s="4" t="n"/>
-      <c r="P6" s="4" t="n"/>
-      <c r="Q6" s="4" t="n"/>
-      <c r="R6" s="4" t="n"/>
-      <c r="S6" s="6" t="inlineStr">
+      <c r="O6" s="6" t="n"/>
+      <c r="P6" s="6" t="n"/>
+      <c r="Q6" s="5" t="n"/>
+      <c r="R6" s="5" t="n"/>
+      <c r="S6" s="5" t="n"/>
+      <c r="T6" s="5" t="n"/>
+      <c r="U6" s="7" t="inlineStr">
         <is>
           <t>سمت های قبلی:</t>
         </is>
       </c>
-      <c r="T6" s="6" t="n"/>
-      <c r="U6" s="6" t="n"/>
-      <c r="V6" s="6" t="n"/>
-      <c r="W6" s="6" t="n"/>
-      <c r="X6" s="6" t="n"/>
+      <c r="V6" s="7" t="n"/>
+      <c r="W6" s="7" t="n"/>
+      <c r="X6" s="7" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="3" t="n"/>
@@ -881,64 +893,64 @@
       <c r="E7" s="4" t="n"/>
       <c r="F7" s="4" t="n"/>
       <c r="G7" s="4" t="n"/>
-      <c r="H7" s="4" t="n"/>
+      <c r="H7" s="5" t="n"/>
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
-      <c r="N7" s="4" t="n"/>
-      <c r="O7" s="4" t="n"/>
-      <c r="P7" s="4" t="n"/>
-      <c r="Q7" s="4" t="n"/>
-      <c r="R7" s="4" t="n"/>
-      <c r="S7" s="7" t="n"/>
-      <c r="T7" s="7" t="n"/>
-      <c r="U7" s="7" t="n"/>
-      <c r="V7" s="7" t="n"/>
-      <c r="W7" s="7" t="n"/>
-      <c r="X7" s="7" t="n"/>
+      <c r="L7" s="6" t="n"/>
+      <c r="M7" s="6" t="n"/>
+      <c r="N7" s="6" t="n"/>
+      <c r="O7" s="6" t="n"/>
+      <c r="P7" s="6" t="n"/>
+      <c r="Q7" s="5" t="n"/>
+      <c r="R7" s="5" t="n"/>
+      <c r="S7" s="5" t="n"/>
+      <c r="T7" s="5" t="n"/>
+      <c r="U7" s="8" t="n"/>
+      <c r="V7" s="8" t="n"/>
+      <c r="W7" s="8" t="n"/>
+      <c r="X7" s="8" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>کدملی:</t>
-        </is>
-      </c>
+      <c r="B8" s="3" t="n"/>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="3" t="n"/>
-      <c r="E8" s="4" t="n"/>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>کدملی:</t>
+        </is>
+      </c>
       <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="n"/>
-      <c r="H8" s="4" t="n"/>
-      <c r="I8" s="8" t="inlineStr">
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="n"/>
+      <c r="J8" s="5" t="n"/>
+      <c r="K8" s="5" t="n"/>
+      <c r="L8" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="J8" s="8" t="inlineStr">
+      <c r="M8" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="N8" s="6" t="inlineStr">
         <is>
           <t>پست سازمانی</t>
         </is>
       </c>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="5" t="n"/>
-      <c r="N8" s="4" t="n"/>
-      <c r="O8" s="4" t="n"/>
-      <c r="P8" s="4" t="n"/>
-      <c r="Q8" s="4" t="n"/>
-      <c r="R8" s="4" t="n"/>
-      <c r="S8" s="7" t="n"/>
-      <c r="T8" s="7" t="n"/>
-      <c r="U8" s="7" t="n"/>
-      <c r="V8" s="7" t="n"/>
-      <c r="W8" s="7" t="n"/>
-      <c r="X8" s="7" t="n"/>
+      <c r="O8" s="6" t="n"/>
+      <c r="P8" s="6" t="n"/>
+      <c r="Q8" s="5" t="n"/>
+      <c r="R8" s="5" t="n"/>
+      <c r="S8" s="5" t="n"/>
+      <c r="T8" s="5" t="n"/>
+      <c r="U8" s="8" t="n"/>
+      <c r="V8" s="8" t="n"/>
+      <c r="W8" s="8" t="n"/>
+      <c r="X8" s="8" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="B9" s="3" t="n"/>
@@ -947,60 +959,60 @@
       <c r="E9" s="4" t="n"/>
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="4" t="n"/>
-      <c r="H9" s="4" t="n"/>
-      <c r="I9" s="8" t="n"/>
-      <c r="J9" s="8" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="n"/>
       <c r="K9" s="5" t="n"/>
-      <c r="L9" s="5" t="n"/>
-      <c r="M9" s="5" t="n"/>
-      <c r="N9" s="4" t="n"/>
-      <c r="O9" s="4" t="n"/>
-      <c r="P9" s="4" t="n"/>
-      <c r="Q9" s="4" t="n"/>
-      <c r="R9" s="4" t="n"/>
-      <c r="S9" s="7" t="n"/>
-      <c r="T9" s="7" t="n"/>
-      <c r="U9" s="7" t="n"/>
-      <c r="V9" s="7" t="n"/>
-      <c r="W9" s="7" t="n"/>
-      <c r="X9" s="7" t="n"/>
+      <c r="L9" s="9" t="n"/>
+      <c r="M9" s="9" t="n"/>
+      <c r="N9" s="6" t="n"/>
+      <c r="O9" s="6" t="n"/>
+      <c r="P9" s="6" t="n"/>
+      <c r="Q9" s="5" t="n"/>
+      <c r="R9" s="5" t="n"/>
+      <c r="S9" s="5" t="n"/>
+      <c r="T9" s="5" t="n"/>
+      <c r="U9" s="8" t="n"/>
+      <c r="V9" s="8" t="n"/>
+      <c r="W9" s="8" t="n"/>
+      <c r="X9" s="8" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>کدپرسنلی</t>
-        </is>
-      </c>
+      <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="3" t="n"/>
-      <c r="E10" s="4" t="n"/>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>کدپرسنلی</t>
+        </is>
+      </c>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
-      <c r="H10" s="4" t="n"/>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="5" t="n"/>
+      <c r="K10" s="5" t="n"/>
+      <c r="L10" s="6" t="inlineStr">
         <is>
           <t>تعدادفرزندان</t>
         </is>
       </c>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="M10" s="6" t="n"/>
+      <c r="N10" s="6" t="inlineStr">
         <is>
           <t>محل خدمت</t>
         </is>
       </c>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
-      <c r="N10" s="4" t="n"/>
-      <c r="O10" s="4" t="n"/>
-      <c r="P10" s="4" t="n"/>
-      <c r="Q10" s="4" t="n"/>
-      <c r="R10" s="4" t="n"/>
-      <c r="S10" s="7" t="n"/>
-      <c r="T10" s="7" t="n"/>
-      <c r="U10" s="7" t="n"/>
-      <c r="V10" s="7" t="n"/>
-      <c r="W10" s="7" t="n"/>
-      <c r="X10" s="7" t="n"/>
+      <c r="O10" s="6" t="n"/>
+      <c r="P10" s="6" t="n"/>
+      <c r="Q10" s="5" t="n"/>
+      <c r="R10" s="5" t="n"/>
+      <c r="S10" s="5" t="n"/>
+      <c r="T10" s="5" t="n"/>
+      <c r="U10" s="8" t="n"/>
+      <c r="V10" s="8" t="n"/>
+      <c r="W10" s="8" t="n"/>
+      <c r="X10" s="8" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="B11" s="3" t="n"/>
@@ -1009,64 +1021,64 @@
       <c r="E11" s="4" t="n"/>
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
-      <c r="H11" s="4" t="n"/>
+      <c r="H11" s="5" t="n"/>
       <c r="I11" s="5" t="n"/>
       <c r="J11" s="5" t="n"/>
       <c r="K11" s="5" t="n"/>
-      <c r="L11" s="5" t="n"/>
-      <c r="M11" s="5" t="n"/>
-      <c r="N11" s="4" t="n"/>
-      <c r="O11" s="4" t="n"/>
-      <c r="P11" s="4" t="n"/>
-      <c r="Q11" s="4" t="n"/>
-      <c r="R11" s="4" t="n"/>
-      <c r="S11" s="7" t="n"/>
-      <c r="T11" s="7" t="n"/>
-      <c r="U11" s="7" t="n"/>
-      <c r="V11" s="7" t="n"/>
-      <c r="W11" s="7" t="n"/>
-      <c r="X11" s="7" t="n"/>
+      <c r="L11" s="6" t="n"/>
+      <c r="M11" s="6" t="n"/>
+      <c r="N11" s="6" t="n"/>
+      <c r="O11" s="6" t="n"/>
+      <c r="P11" s="6" t="n"/>
+      <c r="Q11" s="5" t="n"/>
+      <c r="R11" s="5" t="n"/>
+      <c r="S11" s="5" t="n"/>
+      <c r="T11" s="5" t="n"/>
+      <c r="U11" s="8" t="n"/>
+      <c r="V11" s="8" t="n"/>
+      <c r="W11" s="8" t="n"/>
+      <c r="X11" s="8" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>تاریخ تولد:</t>
-        </is>
-      </c>
+      <c r="B12" s="3" t="n"/>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="3" t="n"/>
-      <c r="E12" s="4" t="n"/>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>تاریخ تولد:</t>
+        </is>
+      </c>
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
-      <c r="H12" s="4" t="n"/>
-      <c r="I12" s="9" t="inlineStr">
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="n"/>
+      <c r="K12" s="5" t="n"/>
+      <c r="L12" s="10" t="inlineStr">
         <is>
           <t>دختر</t>
         </is>
       </c>
-      <c r="J12" s="10" t="inlineStr">
+      <c r="M12" s="11" t="inlineStr">
         <is>
           <t>پسر</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="N12" s="6" t="inlineStr">
         <is>
           <t>تاریخ شروع به کار</t>
         </is>
       </c>
-      <c r="L12" s="5" t="n"/>
-      <c r="M12" s="5" t="n"/>
-      <c r="N12" s="4" t="n"/>
-      <c r="O12" s="4" t="n"/>
-      <c r="P12" s="4" t="n"/>
-      <c r="Q12" s="4" t="n"/>
-      <c r="R12" s="4" t="n"/>
-      <c r="S12" s="7" t="n"/>
-      <c r="T12" s="7" t="n"/>
-      <c r="U12" s="7" t="n"/>
-      <c r="V12" s="7" t="n"/>
-      <c r="W12" s="7" t="n"/>
-      <c r="X12" s="7" t="n"/>
+      <c r="O12" s="6" t="n"/>
+      <c r="P12" s="6" t="n"/>
+      <c r="Q12" s="5" t="n"/>
+      <c r="R12" s="5" t="n"/>
+      <c r="S12" s="5" t="n"/>
+      <c r="T12" s="5" t="n"/>
+      <c r="U12" s="8" t="n"/>
+      <c r="V12" s="8" t="n"/>
+      <c r="W12" s="8" t="n"/>
+      <c r="X12" s="8" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="B13" s="3" t="n"/>
@@ -1075,60 +1087,60 @@
       <c r="E13" s="4" t="n"/>
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="4" t="n"/>
-      <c r="H13" s="4" t="n"/>
-      <c r="I13" s="9" t="n"/>
-      <c r="J13" s="10" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5" t="n"/>
       <c r="K13" s="5" t="n"/>
-      <c r="L13" s="5" t="n"/>
-      <c r="M13" s="5" t="n"/>
-      <c r="N13" s="4" t="n"/>
-      <c r="O13" s="4" t="n"/>
-      <c r="P13" s="4" t="n"/>
-      <c r="Q13" s="4" t="n"/>
-      <c r="R13" s="4" t="n"/>
-      <c r="S13" s="7" t="n"/>
-      <c r="T13" s="7" t="n"/>
-      <c r="U13" s="7" t="n"/>
-      <c r="V13" s="7" t="n"/>
-      <c r="W13" s="7" t="n"/>
-      <c r="X13" s="7" t="n"/>
+      <c r="L13" s="10" t="n"/>
+      <c r="M13" s="11" t="n"/>
+      <c r="N13" s="6" t="n"/>
+      <c r="O13" s="6" t="n"/>
+      <c r="P13" s="6" t="n"/>
+      <c r="Q13" s="5" t="n"/>
+      <c r="R13" s="5" t="n"/>
+      <c r="S13" s="5" t="n"/>
+      <c r="T13" s="5" t="n"/>
+      <c r="U13" s="8" t="n"/>
+      <c r="V13" s="8" t="n"/>
+      <c r="W13" s="8" t="n"/>
+      <c r="X13" s="8" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>مدرک تحصیلی</t>
-        </is>
-      </c>
+      <c r="B14" s="3" t="n"/>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="3" t="n"/>
-      <c r="E14" s="4" t="n"/>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>مدرک تحصیلی</t>
+        </is>
+      </c>
       <c r="F14" s="4" t="n"/>
       <c r="G14" s="4" t="n"/>
-      <c r="H14" s="4" t="n"/>
-      <c r="I14" s="4" t="n"/>
-      <c r="J14" s="4" t="n"/>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t>سوابق خدمتی/تجربی</t>
-        </is>
-      </c>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="n"/>
+      <c r="K14" s="5" t="n"/>
       <c r="L14" s="5" t="n"/>
       <c r="M14" s="5" t="n"/>
-      <c r="N14" s="4" t="n"/>
-      <c r="O14" s="4" t="n"/>
-      <c r="P14" s="4" t="n"/>
-      <c r="Q14" s="4" t="n"/>
-      <c r="R14" s="4" t="n"/>
-      <c r="S14" s="6" t="inlineStr">
+      <c r="N14" s="6" t="inlineStr">
+        <is>
+          <t>سوابق خدمتی/تجربی</t>
+        </is>
+      </c>
+      <c r="O14" s="6" t="n"/>
+      <c r="P14" s="6" t="n"/>
+      <c r="Q14" s="5" t="n"/>
+      <c r="R14" s="5" t="n"/>
+      <c r="S14" s="5" t="n"/>
+      <c r="T14" s="5" t="n"/>
+      <c r="U14" s="7" t="inlineStr">
         <is>
           <t>توقف پست:</t>
         </is>
       </c>
-      <c r="T14" s="6" t="n"/>
-      <c r="U14" s="6" t="n"/>
-      <c r="V14" s="6" t="n"/>
-      <c r="W14" s="6" t="n"/>
-      <c r="X14" s="6" t="n"/>
+      <c r="V14" s="7" t="n"/>
+      <c r="W14" s="7" t="n"/>
+      <c r="X14" s="7" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="B15" s="3" t="n"/>
@@ -1137,56 +1149,56 @@
       <c r="E15" s="4" t="n"/>
       <c r="F15" s="4" t="n"/>
       <c r="G15" s="4" t="n"/>
-      <c r="H15" s="4" t="n"/>
-      <c r="I15" s="4" t="n"/>
-      <c r="J15" s="4" t="n"/>
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
       <c r="K15" s="5" t="n"/>
       <c r="L15" s="5" t="n"/>
       <c r="M15" s="5" t="n"/>
-      <c r="N15" s="4" t="n"/>
-      <c r="O15" s="4" t="n"/>
-      <c r="P15" s="4" t="n"/>
-      <c r="Q15" s="4" t="n"/>
-      <c r="R15" s="4" t="n"/>
-      <c r="S15" s="7" t="n"/>
-      <c r="T15" s="7" t="n"/>
-      <c r="U15" s="7" t="n"/>
-      <c r="V15" s="7" t="n"/>
-      <c r="W15" s="7" t="n"/>
-      <c r="X15" s="7" t="n"/>
+      <c r="N15" s="6" t="n"/>
+      <c r="O15" s="6" t="n"/>
+      <c r="P15" s="6" t="n"/>
+      <c r="Q15" s="5" t="n"/>
+      <c r="R15" s="5" t="n"/>
+      <c r="S15" s="5" t="n"/>
+      <c r="T15" s="5" t="n"/>
+      <c r="U15" s="8" t="n"/>
+      <c r="V15" s="8" t="n"/>
+      <c r="W15" s="8" t="n"/>
+      <c r="X15" s="8" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>رشته تحصیلی</t>
-        </is>
-      </c>
+      <c r="B16" s="3" t="n"/>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="n"/>
-      <c r="E16" s="4" t="n"/>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>رشته تحصیلی</t>
+        </is>
+      </c>
       <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="n"/>
-      <c r="H16" s="4" t="n"/>
-      <c r="I16" s="4" t="n"/>
-      <c r="J16" s="4" t="n"/>
-      <c r="K16" s="5" t="inlineStr">
-        <is>
-          <t>سوابق آموزشی</t>
-        </is>
-      </c>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
+      <c r="K16" s="5" t="n"/>
       <c r="L16" s="5" t="n"/>
       <c r="M16" s="5" t="n"/>
-      <c r="N16" s="4" t="n"/>
-      <c r="O16" s="4" t="n"/>
-      <c r="P16" s="4" t="n"/>
-      <c r="Q16" s="4" t="n"/>
-      <c r="R16" s="4" t="n"/>
-      <c r="S16" s="7" t="n"/>
-      <c r="T16" s="7" t="n"/>
-      <c r="U16" s="7" t="n"/>
-      <c r="V16" s="7" t="n"/>
-      <c r="W16" s="7" t="n"/>
-      <c r="X16" s="7" t="n"/>
+      <c r="N16" s="6" t="inlineStr">
+        <is>
+          <t>سوابق آموزشی</t>
+        </is>
+      </c>
+      <c r="O16" s="6" t="n"/>
+      <c r="P16" s="6" t="n"/>
+      <c r="Q16" s="5" t="n"/>
+      <c r="R16" s="5" t="n"/>
+      <c r="S16" s="5" t="n"/>
+      <c r="T16" s="5" t="n"/>
+      <c r="U16" s="8" t="n"/>
+      <c r="V16" s="8" t="n"/>
+      <c r="W16" s="8" t="n"/>
+      <c r="X16" s="8" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="B17" s="3" t="n"/>
@@ -1195,64 +1207,64 @@
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="4" t="n"/>
       <c r="G17" s="4" t="n"/>
-      <c r="H17" s="4" t="n"/>
-      <c r="I17" s="4" t="n"/>
-      <c r="J17" s="4" t="n"/>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="5" t="n"/>
+      <c r="J17" s="5" t="n"/>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="5" t="n"/>
       <c r="M17" s="5" t="n"/>
-      <c r="N17" s="4" t="n"/>
-      <c r="O17" s="4" t="n"/>
-      <c r="P17" s="4" t="n"/>
-      <c r="Q17" s="4" t="n"/>
-      <c r="R17" s="4" t="n"/>
-      <c r="S17" s="7" t="n"/>
-      <c r="T17" s="7" t="n"/>
-      <c r="U17" s="7" t="n"/>
-      <c r="V17" s="7" t="n"/>
-      <c r="W17" s="7" t="n"/>
-      <c r="X17" s="7" t="n"/>
+      <c r="N17" s="6" t="n"/>
+      <c r="O17" s="6" t="n"/>
+      <c r="P17" s="6" t="n"/>
+      <c r="Q17" s="5" t="n"/>
+      <c r="R17" s="5" t="n"/>
+      <c r="S17" s="5" t="n"/>
+      <c r="T17" s="5" t="n"/>
+      <c r="U17" s="8" t="n"/>
+      <c r="V17" s="8" t="n"/>
+      <c r="W17" s="8" t="n"/>
+      <c r="X17" s="8" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>شماره تماس:</t>
-        </is>
-      </c>
+      <c r="B18" s="3" t="n"/>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="3" t="n"/>
-      <c r="E18" s="4" t="n"/>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>شماره تماس:</t>
+        </is>
+      </c>
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
-      <c r="H18" s="4" t="n"/>
-      <c r="I18" s="4" t="n"/>
-      <c r="J18" s="4" t="n"/>
-      <c r="K18" s="5" t="inlineStr">
-        <is>
-          <t>سوابق ارزیابی</t>
-        </is>
-      </c>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="n"/>
+      <c r="K18" s="5" t="n"/>
       <c r="L18" s="5" t="n"/>
       <c r="M18" s="5" t="n"/>
-      <c r="N18" s="11" t="inlineStr">
+      <c r="N18" s="6" t="inlineStr">
+        <is>
+          <t>سوابق ارزیابی</t>
+        </is>
+      </c>
+      <c r="O18" s="6" t="n"/>
+      <c r="P18" s="6" t="n"/>
+      <c r="Q18" s="12" t="inlineStr">
         <is>
           <t>تنبیهات</t>
         </is>
       </c>
-      <c r="O18" s="11" t="n"/>
-      <c r="P18" s="11" t="inlineStr">
+      <c r="R18" s="12" t="n"/>
+      <c r="S18" s="12" t="inlineStr">
         <is>
           <t>تشویق ها</t>
         </is>
       </c>
-      <c r="Q18" s="11" t="n"/>
-      <c r="R18" s="11" t="n"/>
-      <c r="S18" s="7" t="n"/>
-      <c r="T18" s="7" t="n"/>
-      <c r="U18" s="7" t="n"/>
-      <c r="V18" s="7" t="n"/>
-      <c r="W18" s="7" t="n"/>
-      <c r="X18" s="7" t="n"/>
+      <c r="T18" s="12" t="n"/>
+      <c r="U18" s="8" t="n"/>
+      <c r="V18" s="8" t="n"/>
+      <c r="W18" s="8" t="n"/>
+      <c r="X18" s="8" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="B19" s="3" t="n"/>
@@ -1261,23 +1273,23 @@
       <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="n"/>
       <c r="G19" s="4" t="n"/>
-      <c r="H19" s="4" t="n"/>
-      <c r="I19" s="4" t="n"/>
-      <c r="J19" s="4" t="n"/>
+      <c r="H19" s="5" t="n"/>
+      <c r="I19" s="5" t="n"/>
+      <c r="J19" s="5" t="n"/>
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="5" t="n"/>
       <c r="M19" s="5" t="n"/>
-      <c r="N19" s="4" t="n"/>
-      <c r="O19" s="4" t="n"/>
-      <c r="P19" s="4" t="n"/>
-      <c r="Q19" s="4" t="n"/>
-      <c r="R19" s="4" t="n"/>
-      <c r="S19" s="7" t="n"/>
-      <c r="T19" s="7" t="n"/>
-      <c r="U19" s="7" t="n"/>
-      <c r="V19" s="7" t="n"/>
-      <c r="W19" s="7" t="n"/>
-      <c r="X19" s="7" t="n"/>
+      <c r="N19" s="6" t="n"/>
+      <c r="O19" s="6" t="n"/>
+      <c r="P19" s="6" t="n"/>
+      <c r="Q19" s="5" t="n"/>
+      <c r="R19" s="5" t="n"/>
+      <c r="S19" s="5" t="n"/>
+      <c r="T19" s="5" t="n"/>
+      <c r="U19" s="8" t="n"/>
+      <c r="V19" s="8" t="n"/>
+      <c r="W19" s="8" t="n"/>
+      <c r="X19" s="8" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="B20" s="2" t="inlineStr">
@@ -1335,784 +1347,784 @@
     </row>
     <row r="22" ht="26" customHeight="1"/>
     <row r="23" ht="26" customHeight="1">
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>ارزیابی توانمندی وشایستگی</t>
         </is>
       </c>
-      <c r="C23" s="12" t="n"/>
-      <c r="D23" s="12" t="n"/>
-      <c r="E23" s="12" t="n"/>
-      <c r="F23" s="12" t="n"/>
-      <c r="G23" s="12" t="n"/>
-      <c r="H23" s="12" t="n"/>
-      <c r="I23" s="12" t="n"/>
-      <c r="K23" s="12" t="inlineStr">
+      <c r="C23" s="13" t="n"/>
+      <c r="D23" s="13" t="n"/>
+      <c r="E23" s="13" t="n"/>
+      <c r="F23" s="13" t="n"/>
+      <c r="G23" s="13" t="n"/>
+      <c r="H23" s="13" t="n"/>
+      <c r="I23" s="13" t="n"/>
+      <c r="K23" s="13" t="inlineStr">
         <is>
           <t>کارنامه نظم وانضباط اداری</t>
         </is>
       </c>
-      <c r="L23" s="12" t="n"/>
-      <c r="M23" s="12" t="n"/>
-      <c r="N23" s="12" t="n"/>
-      <c r="O23" s="12" t="n"/>
-      <c r="P23" s="12" t="n"/>
-      <c r="Q23" s="12" t="n"/>
-      <c r="R23" s="12" t="n"/>
-      <c r="S23" s="12" t="n"/>
-      <c r="U23" s="13" t="inlineStr">
+      <c r="L23" s="13" t="n"/>
+      <c r="M23" s="13" t="n"/>
+      <c r="N23" s="13" t="n"/>
+      <c r="O23" s="13" t="n"/>
+      <c r="P23" s="13" t="n"/>
+      <c r="Q23" s="13" t="n"/>
+      <c r="R23" s="13" t="n"/>
+      <c r="S23" s="13" t="n"/>
+      <c r="U23" s="14" t="inlineStr">
         <is>
           <t>جمع بندی وپیشنهادات مدیریتی</t>
         </is>
       </c>
-      <c r="V23" s="13" t="n"/>
-      <c r="W23" s="13" t="n"/>
-      <c r="X23" s="13" t="n"/>
+      <c r="V23" s="14" t="n"/>
+      <c r="W23" s="14" t="n"/>
+      <c r="X23" s="14" t="n"/>
     </row>
     <row r="24" ht="26" customHeight="1">
-      <c r="B24" s="14" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>ردیف</t>
         </is>
       </c>
-      <c r="C24" s="14" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr">
         <is>
           <t>شاخص</t>
         </is>
       </c>
-      <c r="D24" s="14" t="n"/>
-      <c r="E24" s="14" t="n"/>
-      <c r="F24" s="14" t="inlineStr">
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="15" t="inlineStr">
         <is>
           <t>نمره</t>
         </is>
       </c>
-      <c r="G24" s="14" t="inlineStr">
+      <c r="G24" s="15" t="inlineStr">
         <is>
           <t>شرح</t>
         </is>
       </c>
-      <c r="H24" s="14" t="n"/>
-      <c r="I24" s="14" t="n"/>
-      <c r="K24" s="14" t="inlineStr">
+      <c r="H24" s="15" t="n"/>
+      <c r="I24" s="15" t="n"/>
+      <c r="K24" s="15" t="inlineStr">
         <is>
           <t>ردیف</t>
         </is>
       </c>
-      <c r="L24" s="14" t="inlineStr">
+      <c r="L24" s="15" t="inlineStr">
         <is>
           <t>شاخص</t>
         </is>
       </c>
-      <c r="M24" s="14" t="n"/>
-      <c r="N24" s="14" t="n"/>
-      <c r="O24" s="14" t="inlineStr">
+      <c r="M24" s="15" t="n"/>
+      <c r="N24" s="15" t="n"/>
+      <c r="O24" s="15" t="inlineStr">
         <is>
           <t>نمره</t>
         </is>
       </c>
-      <c r="P24" s="14" t="inlineStr">
+      <c r="P24" s="15" t="inlineStr">
         <is>
           <t>توضیحات/مستندات</t>
         </is>
       </c>
-      <c r="Q24" s="14" t="n"/>
-      <c r="R24" s="14" t="n"/>
-      <c r="S24" s="14" t="n"/>
-      <c r="U24" s="15" t="inlineStr">
+      <c r="Q24" s="15" t="n"/>
+      <c r="R24" s="15" t="n"/>
+      <c r="S24" s="15" t="n"/>
+      <c r="U24" s="16" t="inlineStr">
         <is>
           <t>شایسته تقدیروتشویق</t>
         </is>
       </c>
-      <c r="V24" s="15" t="n"/>
-      <c r="W24" s="16" t="inlineStr">
+      <c r="V24" s="16" t="n"/>
+      <c r="W24" s="17" t="inlineStr">
         <is>
           <t>✸</t>
         </is>
       </c>
-      <c r="X24" s="17" t="inlineStr">
+      <c r="X24" s="18" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
     </row>
     <row r="25" ht="26" customHeight="1">
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>۱</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>تخصص وتسلط بروظایف</t>
         </is>
       </c>
-      <c r="D25" s="4" t="n"/>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="15" t="n"/>
-      <c r="H25" s="15" t="n"/>
-      <c r="I25" s="15" t="n"/>
-      <c r="K25" s="4" t="inlineStr">
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="16" t="n"/>
+      <c r="H25" s="16" t="n"/>
+      <c r="I25" s="16" t="n"/>
+      <c r="K25" s="5" t="inlineStr">
         <is>
           <t>۱</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="L25" s="5" t="inlineStr">
         <is>
           <t>ورود وخروج به موقع</t>
         </is>
       </c>
-      <c r="M25" s="4" t="n"/>
-      <c r="N25" s="4" t="n"/>
-      <c r="O25" s="4" t="n"/>
-      <c r="P25" s="15" t="n"/>
-      <c r="Q25" s="15" t="n"/>
-      <c r="R25" s="15" t="n"/>
-      <c r="S25" s="15" t="n"/>
-      <c r="U25" s="15" t="inlineStr">
+      <c r="M25" s="5" t="n"/>
+      <c r="N25" s="5" t="n"/>
+      <c r="O25" s="5" t="n"/>
+      <c r="P25" s="16" t="n"/>
+      <c r="Q25" s="16" t="n"/>
+      <c r="R25" s="16" t="n"/>
+      <c r="S25" s="16" t="n"/>
+      <c r="U25" s="16" t="inlineStr">
         <is>
           <t>مناسب استمراردرمسئولیت فعلی</t>
         </is>
       </c>
-      <c r="V25" s="15" t="n"/>
-      <c r="W25" s="18" t="inlineStr">
+      <c r="V25" s="16" t="n"/>
+      <c r="W25" s="19" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="X25" s="17" t="inlineStr">
+      <c r="X25" s="18" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
     </row>
     <row r="26" ht="26" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>۲</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>دقت وکیفیت انجام کار</t>
         </is>
       </c>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="15" t="n"/>
-      <c r="H26" s="15" t="n"/>
-      <c r="I26" s="15" t="n"/>
-      <c r="K26" s="4" t="inlineStr">
+      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="5" t="n"/>
+      <c r="F26" s="5" t="n"/>
+      <c r="G26" s="16" t="n"/>
+      <c r="H26" s="16" t="n"/>
+      <c r="I26" s="16" t="n"/>
+      <c r="K26" s="5" t="inlineStr">
         <is>
           <t>۲</t>
         </is>
       </c>
-      <c r="L26" s="4" t="inlineStr">
+      <c r="L26" s="5" t="inlineStr">
         <is>
           <t>میزان تأخیر/غیبت غیرموجه</t>
         </is>
       </c>
-      <c r="M26" s="4" t="n"/>
-      <c r="N26" s="4" t="n"/>
-      <c r="O26" s="4" t="n"/>
-      <c r="P26" s="15" t="n"/>
-      <c r="Q26" s="15" t="n"/>
-      <c r="R26" s="15" t="n"/>
-      <c r="S26" s="15" t="n"/>
-      <c r="U26" s="15" t="inlineStr">
+      <c r="M26" s="5" t="n"/>
+      <c r="N26" s="5" t="n"/>
+      <c r="O26" s="5" t="n"/>
+      <c r="P26" s="16" t="n"/>
+      <c r="Q26" s="16" t="n"/>
+      <c r="R26" s="16" t="n"/>
+      <c r="S26" s="16" t="n"/>
+      <c r="U26" s="16" t="inlineStr">
         <is>
           <t>شایسته ارتقای شغلی</t>
         </is>
       </c>
-      <c r="V26" s="15" t="n"/>
-      <c r="W26" s="19" t="inlineStr">
+      <c r="V26" s="16" t="n"/>
+      <c r="W26" s="20" t="inlineStr">
         <is>
           <t>⚑</t>
         </is>
       </c>
-      <c r="X26" s="17" t="inlineStr">
+      <c r="X26" s="18" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
     </row>
     <row r="27" ht="26" customHeight="1">
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>۳</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>مسئولیت پذیری</t>
         </is>
       </c>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="15" t="n"/>
-      <c r="H27" s="15" t="n"/>
-      <c r="I27" s="15" t="n"/>
-      <c r="K27" s="4" t="inlineStr">
+      <c r="D27" s="5" t="n"/>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
+      <c r="G27" s="16" t="n"/>
+      <c r="H27" s="16" t="n"/>
+      <c r="I27" s="16" t="n"/>
+      <c r="K27" s="5" t="inlineStr">
         <is>
           <t>۳</t>
         </is>
       </c>
-      <c r="L27" s="4" t="inlineStr">
+      <c r="L27" s="5" t="inlineStr">
         <is>
           <t>رعایت شئونات اداری</t>
         </is>
       </c>
-      <c r="M27" s="4" t="n"/>
-      <c r="N27" s="4" t="n"/>
-      <c r="O27" s="4" t="n"/>
-      <c r="P27" s="15" t="n"/>
-      <c r="Q27" s="15" t="n"/>
-      <c r="R27" s="15" t="n"/>
-      <c r="S27" s="15" t="n"/>
-      <c r="U27" s="15" t="inlineStr">
+      <c r="M27" s="5" t="n"/>
+      <c r="N27" s="5" t="n"/>
+      <c r="O27" s="5" t="n"/>
+      <c r="P27" s="16" t="n"/>
+      <c r="Q27" s="16" t="n"/>
+      <c r="R27" s="16" t="n"/>
+      <c r="S27" s="16" t="n"/>
+      <c r="U27" s="16" t="inlineStr">
         <is>
           <t>مستعدپذیرش مسئولیت بالاتر</t>
         </is>
       </c>
-      <c r="V27" s="15" t="n"/>
-      <c r="W27" s="20" t="inlineStr">
+      <c r="V27" s="16" t="n"/>
+      <c r="W27" s="21" t="inlineStr">
         <is>
           <t>☁</t>
         </is>
       </c>
-      <c r="X27" s="17" t="inlineStr">
+      <c r="X27" s="18" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
     </row>
     <row r="28" ht="26" customHeight="1">
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>۴</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>توانائی حل مسئله ومدیریت امور</t>
         </is>
       </c>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="15" t="n"/>
-      <c r="H28" s="15" t="n"/>
-      <c r="I28" s="15" t="n"/>
-      <c r="K28" s="4" t="inlineStr">
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
+      <c r="G28" s="16" t="n"/>
+      <c r="H28" s="16" t="n"/>
+      <c r="I28" s="16" t="n"/>
+      <c r="K28" s="5" t="inlineStr">
         <is>
           <t>۴</t>
         </is>
       </c>
-      <c r="L28" s="4" t="inlineStr">
+      <c r="L28" s="5" t="inlineStr">
         <is>
           <t>پایبندی به اصول اخلاق حرفه ای</t>
         </is>
       </c>
-      <c r="M28" s="4" t="n"/>
-      <c r="N28" s="4" t="n"/>
-      <c r="O28" s="4" t="n"/>
-      <c r="P28" s="15" t="n"/>
-      <c r="Q28" s="15" t="n"/>
-      <c r="R28" s="15" t="n"/>
-      <c r="S28" s="15" t="n"/>
-      <c r="U28" s="15" t="inlineStr">
+      <c r="M28" s="5" t="n"/>
+      <c r="N28" s="5" t="n"/>
+      <c r="O28" s="5" t="n"/>
+      <c r="P28" s="16" t="n"/>
+      <c r="Q28" s="16" t="n"/>
+      <c r="R28" s="16" t="n"/>
+      <c r="S28" s="16" t="n"/>
+      <c r="U28" s="16" t="inlineStr">
         <is>
           <t>نیازمندبرنامه بهبودعملکرد</t>
         </is>
       </c>
-      <c r="V28" s="15" t="n"/>
-      <c r="W28" s="21" t="inlineStr">
+      <c r="V28" s="16" t="n"/>
+      <c r="W28" s="22" t="inlineStr">
         <is>
           <t>■</t>
         </is>
       </c>
-      <c r="X28" s="17" t="inlineStr">
+      <c r="X28" s="18" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1">
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>۵</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>همکاری وکارتیمی</t>
         </is>
       </c>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="15" t="n"/>
-      <c r="H29" s="15" t="n"/>
-      <c r="I29" s="15" t="n"/>
-      <c r="K29" s="4" t="inlineStr">
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="16" t="n"/>
+      <c r="H29" s="16" t="n"/>
+      <c r="I29" s="16" t="n"/>
+      <c r="K29" s="5" t="inlineStr">
         <is>
           <t>۵</t>
         </is>
       </c>
-      <c r="L29" s="4" t="inlineStr">
+      <c r="L29" s="5" t="inlineStr">
         <is>
           <t>آراستگی وپوشش</t>
         </is>
       </c>
-      <c r="M29" s="4" t="n"/>
-      <c r="N29" s="4" t="n"/>
-      <c r="O29" s="4" t="n"/>
-      <c r="P29" s="15" t="n"/>
-      <c r="Q29" s="15" t="n"/>
-      <c r="R29" s="15" t="n"/>
-      <c r="S29" s="15" t="n"/>
-      <c r="U29" s="15" t="inlineStr">
+      <c r="M29" s="5" t="n"/>
+      <c r="N29" s="5" t="n"/>
+      <c r="O29" s="5" t="n"/>
+      <c r="P29" s="16" t="n"/>
+      <c r="Q29" s="16" t="n"/>
+      <c r="R29" s="16" t="n"/>
+      <c r="S29" s="16" t="n"/>
+      <c r="U29" s="16" t="inlineStr">
         <is>
           <t>نیازمندبررسی مجددمسئولیت</t>
         </is>
       </c>
-      <c r="V29" s="15" t="n"/>
-      <c r="W29" s="21" t="inlineStr">
+      <c r="V29" s="16" t="n"/>
+      <c r="W29" s="22" t="inlineStr">
         <is>
           <t>■</t>
         </is>
       </c>
-      <c r="X29" s="17" t="inlineStr">
+      <c r="X29" s="18" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
     </row>
     <row r="30" ht="26" customHeight="1">
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>۶</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>تعامل وارتباط مؤثر</t>
         </is>
       </c>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="n"/>
-      <c r="G30" s="15" t="n"/>
-      <c r="H30" s="15" t="n"/>
-      <c r="I30" s="15" t="n"/>
-      <c r="K30" s="4" t="inlineStr">
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="16" t="n"/>
+      <c r="H30" s="16" t="n"/>
+      <c r="I30" s="16" t="n"/>
+      <c r="K30" s="5" t="inlineStr">
         <is>
           <t>۶</t>
         </is>
       </c>
-      <c r="L30" s="4" t="inlineStr">
+      <c r="L30" s="5" t="inlineStr">
         <is>
           <t>شرکت درمراسم مذهبی_فرهنگی</t>
         </is>
       </c>
-      <c r="M30" s="4" t="n"/>
-      <c r="N30" s="4" t="n"/>
-      <c r="O30" s="4" t="n"/>
-      <c r="P30" s="15" t="n"/>
-      <c r="Q30" s="15" t="n"/>
-      <c r="R30" s="15" t="n"/>
-      <c r="S30" s="15" t="n"/>
-      <c r="U30" s="3" t="inlineStr">
+      <c r="M30" s="5" t="n"/>
+      <c r="N30" s="5" t="n"/>
+      <c r="O30" s="5" t="n"/>
+      <c r="P30" s="16" t="n"/>
+      <c r="Q30" s="16" t="n"/>
+      <c r="R30" s="16" t="n"/>
+      <c r="S30" s="16" t="n"/>
+      <c r="U30" s="4" t="inlineStr">
         <is>
           <t>توضیحات تکمیلی:</t>
         </is>
       </c>
-      <c r="V30" s="3" t="n"/>
-      <c r="W30" s="3" t="n"/>
-      <c r="X30" s="3" t="n"/>
+      <c r="V30" s="4" t="n"/>
+      <c r="W30" s="4" t="n"/>
+      <c r="X30" s="4" t="n"/>
     </row>
     <row r="31" ht="26" customHeight="1">
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>۷</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>ابتکاروارائه پیشنهادموثر</t>
         </is>
       </c>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="15" t="n"/>
-      <c r="H31" s="15" t="n"/>
-      <c r="I31" s="15" t="n"/>
-      <c r="K31" s="4" t="inlineStr">
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="16" t="n"/>
+      <c r="H31" s="16" t="n"/>
+      <c r="I31" s="16" t="n"/>
+      <c r="K31" s="5" t="inlineStr">
         <is>
           <t>۷</t>
         </is>
       </c>
-      <c r="L31" s="4" t="inlineStr">
+      <c r="L31" s="5" t="inlineStr">
         <is>
           <t>تعهدات وتذکرات</t>
         </is>
       </c>
-      <c r="M31" s="4" t="n"/>
-      <c r="N31" s="4" t="n"/>
-      <c r="O31" s="22" t="inlineStr">
+      <c r="M31" s="5" t="n"/>
+      <c r="N31" s="5" t="n"/>
+      <c r="O31" s="23" t="inlineStr">
         <is>
           <t>تذکر</t>
         </is>
       </c>
-      <c r="P31" s="15" t="n"/>
-      <c r="Q31" s="15" t="n"/>
-      <c r="R31" s="15" t="n"/>
-      <c r="S31" s="15" t="n"/>
-      <c r="U31" s="23" t="n"/>
-      <c r="V31" s="23" t="n"/>
-      <c r="W31" s="23" t="n"/>
-      <c r="X31" s="23" t="n"/>
+      <c r="P31" s="16" t="n"/>
+      <c r="Q31" s="16" t="n"/>
+      <c r="R31" s="16" t="n"/>
+      <c r="S31" s="16" t="n"/>
+      <c r="U31" s="24" t="n"/>
+      <c r="V31" s="24" t="n"/>
+      <c r="W31" s="24" t="n"/>
+      <c r="X31" s="24" t="n"/>
     </row>
     <row r="32" ht="26" customHeight="1">
-      <c r="B32" s="24" t="inlineStr">
+      <c r="B32" s="25" t="inlineStr">
         <is>
           <t>جمع امتیاز</t>
         </is>
       </c>
-      <c r="C32" s="24" t="n"/>
-      <c r="D32" s="24" t="n"/>
-      <c r="E32" s="24" t="n"/>
-      <c r="F32" s="5" t="n"/>
-      <c r="G32" s="25" t="n"/>
-      <c r="H32" s="25" t="n"/>
-      <c r="I32" s="25" t="n"/>
-      <c r="K32" s="4" t="n"/>
-      <c r="L32" s="4" t="n"/>
-      <c r="M32" s="4" t="n"/>
-      <c r="N32" s="4" t="n"/>
-      <c r="O32" s="26" t="inlineStr">
+      <c r="C32" s="25" t="n"/>
+      <c r="D32" s="25" t="n"/>
+      <c r="E32" s="25" t="n"/>
+      <c r="F32" s="6" t="n"/>
+      <c r="G32" s="26" t="n"/>
+      <c r="H32" s="26" t="n"/>
+      <c r="I32" s="26" t="n"/>
+      <c r="K32" s="5" t="n"/>
+      <c r="L32" s="5" t="n"/>
+      <c r="M32" s="5" t="n"/>
+      <c r="N32" s="5" t="n"/>
+      <c r="O32" s="27" t="inlineStr">
         <is>
           <t>تعهد</t>
         </is>
       </c>
-      <c r="P32" s="15" t="n"/>
-      <c r="Q32" s="15" t="n"/>
-      <c r="R32" s="15" t="n"/>
-      <c r="S32" s="15" t="n"/>
-      <c r="U32" s="23" t="n"/>
-      <c r="V32" s="23" t="n"/>
-      <c r="W32" s="23" t="n"/>
-      <c r="X32" s="23" t="n"/>
+      <c r="P32" s="16" t="n"/>
+      <c r="Q32" s="16" t="n"/>
+      <c r="R32" s="16" t="n"/>
+      <c r="S32" s="16" t="n"/>
+      <c r="U32" s="24" t="n"/>
+      <c r="V32" s="24" t="n"/>
+      <c r="W32" s="24" t="n"/>
+      <c r="X32" s="24" t="n"/>
     </row>
     <row r="33" ht="26" customHeight="1">
-      <c r="B33" s="24" t="n"/>
-      <c r="C33" s="24" t="n"/>
-      <c r="D33" s="24" t="n"/>
-      <c r="E33" s="24" t="n"/>
-      <c r="F33" s="5" t="n"/>
-      <c r="G33" s="25" t="n"/>
-      <c r="H33" s="25" t="n"/>
-      <c r="I33" s="25" t="n"/>
-      <c r="K33" s="4" t="n"/>
-      <c r="L33" s="4" t="n"/>
-      <c r="M33" s="4" t="n"/>
-      <c r="N33" s="4" t="n"/>
-      <c r="O33" s="26" t="n"/>
-      <c r="P33" s="15" t="n"/>
-      <c r="Q33" s="15" t="n"/>
-      <c r="R33" s="15" t="n"/>
-      <c r="S33" s="15" t="n"/>
-      <c r="U33" s="23" t="n"/>
-      <c r="V33" s="23" t="n"/>
-      <c r="W33" s="23" t="n"/>
-      <c r="X33" s="23" t="n"/>
+      <c r="B33" s="25" t="n"/>
+      <c r="C33" s="25" t="n"/>
+      <c r="D33" s="25" t="n"/>
+      <c r="E33" s="25" t="n"/>
+      <c r="F33" s="6" t="n"/>
+      <c r="G33" s="26" t="n"/>
+      <c r="H33" s="26" t="n"/>
+      <c r="I33" s="26" t="n"/>
+      <c r="K33" s="5" t="n"/>
+      <c r="L33" s="5" t="n"/>
+      <c r="M33" s="5" t="n"/>
+      <c r="N33" s="5" t="n"/>
+      <c r="O33" s="27" t="n"/>
+      <c r="P33" s="16" t="n"/>
+      <c r="Q33" s="16" t="n"/>
+      <c r="R33" s="16" t="n"/>
+      <c r="S33" s="16" t="n"/>
+      <c r="U33" s="24" t="n"/>
+      <c r="V33" s="24" t="n"/>
+      <c r="W33" s="24" t="n"/>
+      <c r="X33" s="24" t="n"/>
     </row>
     <row r="34" ht="26" customHeight="1"/>
     <row r="35" ht="26" customHeight="1">
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>سوابق ارزیابی ۵ سال گذشته</t>
         </is>
       </c>
-      <c r="C35" s="12" t="n"/>
-      <c r="D35" s="12" t="n"/>
-      <c r="E35" s="12" t="n"/>
-      <c r="F35" s="12" t="n"/>
-      <c r="G35" s="12" t="n"/>
-      <c r="H35" s="12" t="n"/>
-      <c r="I35" s="12" t="n"/>
-      <c r="K35" s="12" t="inlineStr">
+      <c r="C35" s="13" t="n"/>
+      <c r="D35" s="13" t="n"/>
+      <c r="E35" s="13" t="n"/>
+      <c r="F35" s="13" t="n"/>
+      <c r="G35" s="13" t="n"/>
+      <c r="H35" s="13" t="n"/>
+      <c r="I35" s="13" t="n"/>
+      <c r="K35" s="13" t="inlineStr">
         <is>
           <t>رضایت سنجی</t>
         </is>
       </c>
-      <c r="L35" s="12" t="n"/>
-      <c r="M35" s="12" t="n"/>
-      <c r="N35" s="12" t="n"/>
-      <c r="O35" s="12" t="n"/>
-      <c r="P35" s="12" t="n"/>
-      <c r="Q35" s="12" t="n"/>
-      <c r="R35" s="12" t="n"/>
-      <c r="S35" s="12" t="n"/>
-      <c r="U35" s="13" t="inlineStr">
+      <c r="L35" s="13" t="n"/>
+      <c r="M35" s="13" t="n"/>
+      <c r="N35" s="13" t="n"/>
+      <c r="O35" s="13" t="n"/>
+      <c r="P35" s="13" t="n"/>
+      <c r="Q35" s="13" t="n"/>
+      <c r="R35" s="13" t="n"/>
+      <c r="S35" s="13" t="n"/>
+      <c r="U35" s="14" t="inlineStr">
         <is>
           <t>جمع بندی نهائی ارزیابی عملکرد</t>
         </is>
       </c>
-      <c r="V35" s="13" t="n"/>
-      <c r="W35" s="13" t="n"/>
-      <c r="X35" s="13" t="n"/>
+      <c r="V35" s="14" t="n"/>
+      <c r="W35" s="14" t="n"/>
+      <c r="X35" s="14" t="n"/>
     </row>
     <row r="36" ht="26" customHeight="1">
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>سال</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
+      <c r="C36" s="12" t="inlineStr">
         <is>
           <t>نمره کل</t>
         </is>
       </c>
-      <c r="D36" s="11" t="inlineStr">
+      <c r="D36" s="12" t="inlineStr">
         <is>
           <t>رتبه</t>
         </is>
       </c>
-      <c r="E36" s="11" t="inlineStr">
+      <c r="E36" s="12" t="inlineStr">
         <is>
           <t>روندعملکرد</t>
         </is>
       </c>
-      <c r="F36" s="11" t="n"/>
-      <c r="G36" s="11" t="inlineStr">
+      <c r="F36" s="12" t="n"/>
+      <c r="G36" s="12" t="inlineStr">
         <is>
           <t>نقاط قوت شاخص</t>
         </is>
       </c>
-      <c r="H36" s="11" t="n"/>
-      <c r="I36" s="11" t="inlineStr">
+      <c r="H36" s="12" t="n"/>
+      <c r="I36" s="12" t="inlineStr">
         <is>
           <t>مواردنیازمند بهبود</t>
         </is>
       </c>
-      <c r="K36" s="14" t="inlineStr">
+      <c r="K36" s="15" t="inlineStr">
         <is>
           <t>ردیف</t>
         </is>
       </c>
-      <c r="L36" s="14" t="inlineStr">
+      <c r="L36" s="15" t="inlineStr">
         <is>
           <t>شاخص</t>
         </is>
       </c>
-      <c r="M36" s="14" t="n"/>
-      <c r="N36" s="14" t="n"/>
-      <c r="O36" s="14" t="inlineStr">
+      <c r="M36" s="15" t="n"/>
+      <c r="N36" s="15" t="n"/>
+      <c r="O36" s="15" t="inlineStr">
         <is>
           <t>امتیاز</t>
         </is>
       </c>
-      <c r="P36" s="14" t="inlineStr">
+      <c r="P36" s="15" t="inlineStr">
         <is>
           <t>شرح</t>
         </is>
       </c>
-      <c r="Q36" s="14" t="n"/>
-      <c r="R36" s="14" t="n"/>
-      <c r="S36" s="14" t="n"/>
-      <c r="U36" s="15" t="inlineStr">
+      <c r="Q36" s="15" t="n"/>
+      <c r="R36" s="15" t="n"/>
+      <c r="S36" s="15" t="n"/>
+      <c r="U36" s="16" t="inlineStr">
         <is>
           <t>امتیازعملکردواحد/شعبه</t>
         </is>
       </c>
-      <c r="V36" s="15" t="n"/>
-      <c r="W36" s="15" t="n"/>
-      <c r="X36" s="27" t="n"/>
+      <c r="V36" s="16" t="n"/>
+      <c r="W36" s="16" t="n"/>
+      <c r="X36" s="28" t="n"/>
     </row>
     <row r="37" ht="32" customHeight="1">
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>۱۴۰۰</t>
         </is>
       </c>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
-      <c r="E37" s="28" t="n"/>
-      <c r="F37" s="28" t="n"/>
-      <c r="G37" s="28" t="n"/>
-      <c r="H37" s="28" t="n"/>
-      <c r="I37" s="28" t="n"/>
-      <c r="K37" s="4" t="inlineStr">
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="29" t="n"/>
+      <c r="F37" s="29" t="n"/>
+      <c r="G37" s="29" t="n"/>
+      <c r="H37" s="29" t="n"/>
+      <c r="I37" s="29" t="n"/>
+      <c r="K37" s="5" t="inlineStr">
         <is>
           <t>۱</t>
         </is>
       </c>
-      <c r="L37" s="4" t="inlineStr">
+      <c r="L37" s="5" t="inlineStr">
         <is>
           <t>رضایت مدیرمستقیم</t>
         </is>
       </c>
-      <c r="M37" s="4" t="n"/>
-      <c r="N37" s="4" t="n"/>
-      <c r="O37" s="4" t="n"/>
-      <c r="P37" s="15" t="n"/>
-      <c r="Q37" s="15" t="n"/>
-      <c r="R37" s="15" t="n"/>
-      <c r="S37" s="15" t="n"/>
-      <c r="U37" s="15" t="inlineStr">
+      <c r="M37" s="5" t="n"/>
+      <c r="N37" s="5" t="n"/>
+      <c r="O37" s="5" t="n"/>
+      <c r="P37" s="16" t="n"/>
+      <c r="Q37" s="16" t="n"/>
+      <c r="R37" s="16" t="n"/>
+      <c r="S37" s="16" t="n"/>
+      <c r="U37" s="16" t="inlineStr">
         <is>
           <t>امتیازعملکردفردی</t>
         </is>
       </c>
-      <c r="V37" s="15" t="n"/>
-      <c r="W37" s="15" t="n"/>
-      <c r="X37" s="27" t="n"/>
+      <c r="V37" s="16" t="n"/>
+      <c r="W37" s="16" t="n"/>
+      <c r="X37" s="28" t="n"/>
     </row>
     <row r="38" ht="32" customHeight="1">
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>۱۴۰۱</t>
         </is>
       </c>
-      <c r="C38" s="4" t="n"/>
-      <c r="D38" s="4" t="n"/>
-      <c r="E38" s="28" t="n"/>
-      <c r="F38" s="28" t="n"/>
-      <c r="G38" s="28" t="n"/>
-      <c r="H38" s="28" t="n"/>
-      <c r="I38" s="28" t="n"/>
-      <c r="K38" s="4" t="inlineStr">
+      <c r="C38" s="5" t="n"/>
+      <c r="D38" s="5" t="n"/>
+      <c r="E38" s="29" t="n"/>
+      <c r="F38" s="29" t="n"/>
+      <c r="G38" s="29" t="n"/>
+      <c r="H38" s="29" t="n"/>
+      <c r="I38" s="29" t="n"/>
+      <c r="K38" s="5" t="inlineStr">
         <is>
           <t>۲</t>
         </is>
       </c>
-      <c r="L38" s="4" t="inlineStr">
+      <c r="L38" s="5" t="inlineStr">
         <is>
           <t>رضایت ارباب رجوع</t>
         </is>
       </c>
-      <c r="M38" s="4" t="n"/>
-      <c r="N38" s="4" t="n"/>
-      <c r="O38" s="4" t="n"/>
-      <c r="P38" s="15" t="n"/>
-      <c r="Q38" s="15" t="n"/>
-      <c r="R38" s="15" t="n"/>
-      <c r="S38" s="15" t="n"/>
-      <c r="U38" s="15" t="inlineStr">
+      <c r="M38" s="5" t="n"/>
+      <c r="N38" s="5" t="n"/>
+      <c r="O38" s="5" t="n"/>
+      <c r="P38" s="16" t="n"/>
+      <c r="Q38" s="16" t="n"/>
+      <c r="R38" s="16" t="n"/>
+      <c r="S38" s="16" t="n"/>
+      <c r="U38" s="16" t="inlineStr">
         <is>
           <t>امتیازتوانمندی حرفه ای</t>
         </is>
       </c>
-      <c r="V38" s="15" t="n"/>
-      <c r="W38" s="15" t="n"/>
-      <c r="X38" s="27" t="n"/>
+      <c r="V38" s="16" t="n"/>
+      <c r="W38" s="16" t="n"/>
+      <c r="X38" s="28" t="n"/>
     </row>
     <row r="39" ht="32" customHeight="1">
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>۱۴۰۲</t>
         </is>
       </c>
-      <c r="C39" s="4" t="n"/>
-      <c r="D39" s="4" t="n"/>
-      <c r="E39" s="28" t="n"/>
-      <c r="F39" s="28" t="n"/>
-      <c r="G39" s="28" t="n"/>
-      <c r="H39" s="28" t="n"/>
-      <c r="I39" s="28" t="n"/>
-      <c r="K39" s="29" t="inlineStr">
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="29" t="n"/>
+      <c r="F39" s="29" t="n"/>
+      <c r="G39" s="29" t="n"/>
+      <c r="H39" s="29" t="n"/>
+      <c r="I39" s="29" t="n"/>
+      <c r="K39" s="30" t="inlineStr">
         <is>
           <t>منبع ارزیابی:سامانه سامع/ دفترارتباطات مردمی/مراجعات حضوری/تقدیرهاوشکایات</t>
         </is>
       </c>
-      <c r="L39" s="29" t="n"/>
-      <c r="M39" s="29" t="n"/>
-      <c r="N39" s="29" t="n"/>
-      <c r="O39" s="29" t="n"/>
-      <c r="P39" s="29" t="n"/>
-      <c r="Q39" s="29" t="n"/>
-      <c r="R39" s="29" t="n"/>
-      <c r="S39" s="29" t="n"/>
-      <c r="U39" s="15" t="inlineStr">
+      <c r="L39" s="30" t="n"/>
+      <c r="M39" s="30" t="n"/>
+      <c r="N39" s="30" t="n"/>
+      <c r="O39" s="30" t="n"/>
+      <c r="P39" s="30" t="n"/>
+      <c r="Q39" s="30" t="n"/>
+      <c r="R39" s="30" t="n"/>
+      <c r="S39" s="30" t="n"/>
+      <c r="U39" s="16" t="inlineStr">
         <is>
           <t>امتیازنظم وانضباط اداری</t>
         </is>
       </c>
-      <c r="V39" s="15" t="n"/>
-      <c r="W39" s="15" t="n"/>
-      <c r="X39" s="27" t="n"/>
+      <c r="V39" s="16" t="n"/>
+      <c r="W39" s="16" t="n"/>
+      <c r="X39" s="28" t="n"/>
     </row>
     <row r="40" ht="32" customHeight="1">
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>۱۴۰۳</t>
         </is>
       </c>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="4" t="n"/>
-      <c r="E40" s="28" t="n"/>
-      <c r="F40" s="28" t="n"/>
-      <c r="G40" s="28" t="n"/>
-      <c r="H40" s="28" t="n"/>
-      <c r="I40" s="28" t="n"/>
-      <c r="K40" s="29" t="n"/>
-      <c r="L40" s="29" t="n"/>
-      <c r="M40" s="29" t="n"/>
-      <c r="N40" s="29" t="n"/>
-      <c r="O40" s="29" t="n"/>
-      <c r="P40" s="29" t="n"/>
-      <c r="Q40" s="29" t="n"/>
-      <c r="R40" s="29" t="n"/>
-      <c r="S40" s="29" t="n"/>
-      <c r="U40" s="15" t="inlineStr">
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="5" t="n"/>
+      <c r="E40" s="29" t="n"/>
+      <c r="F40" s="29" t="n"/>
+      <c r="G40" s="29" t="n"/>
+      <c r="H40" s="29" t="n"/>
+      <c r="I40" s="29" t="n"/>
+      <c r="K40" s="30" t="n"/>
+      <c r="L40" s="30" t="n"/>
+      <c r="M40" s="30" t="n"/>
+      <c r="N40" s="30" t="n"/>
+      <c r="O40" s="30" t="n"/>
+      <c r="P40" s="30" t="n"/>
+      <c r="Q40" s="30" t="n"/>
+      <c r="R40" s="30" t="n"/>
+      <c r="S40" s="30" t="n"/>
+      <c r="U40" s="16" t="inlineStr">
         <is>
           <t>امتیازرضایت مدیر</t>
         </is>
       </c>
-      <c r="V40" s="15" t="n"/>
-      <c r="W40" s="15" t="n"/>
-      <c r="X40" s="27" t="n"/>
+      <c r="V40" s="16" t="n"/>
+      <c r="W40" s="16" t="n"/>
+      <c r="X40" s="28" t="n"/>
     </row>
     <row r="41" ht="32" customHeight="1">
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>۱۴۰۴</t>
         </is>
       </c>
-      <c r="C41" s="4" t="n"/>
-      <c r="D41" s="4" t="n"/>
-      <c r="E41" s="28" t="n"/>
-      <c r="F41" s="28" t="n"/>
-      <c r="G41" s="28" t="n"/>
-      <c r="H41" s="28" t="n"/>
-      <c r="I41" s="28" t="n"/>
-      <c r="U41" s="15" t="inlineStr">
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="5" t="n"/>
+      <c r="E41" s="29" t="n"/>
+      <c r="F41" s="29" t="n"/>
+      <c r="G41" s="29" t="n"/>
+      <c r="H41" s="29" t="n"/>
+      <c r="I41" s="29" t="n"/>
+      <c r="U41" s="16" t="inlineStr">
         <is>
           <t>امتیازتکریم ارباب رجوع</t>
         </is>
       </c>
-      <c r="V41" s="15" t="n"/>
-      <c r="W41" s="15" t="n"/>
-      <c r="X41" s="27" t="n"/>
+      <c r="V41" s="16" t="n"/>
+      <c r="W41" s="16" t="n"/>
+      <c r="X41" s="28" t="n"/>
     </row>
     <row r="42" ht="26" customHeight="1">
-      <c r="B42" s="14" t="inlineStr">
+      <c r="B42" s="15" t="inlineStr">
         <is>
           <t>میانگین ۵ ساله</t>
         </is>
       </c>
-      <c r="C42" s="14" t="n"/>
-      <c r="D42" s="14" t="n"/>
-      <c r="E42" s="5" t="n"/>
-      <c r="F42" s="5" t="n"/>
-      <c r="G42" s="5" t="n"/>
-      <c r="H42" s="5" t="n"/>
-      <c r="I42" s="5" t="n"/>
+      <c r="C42" s="15" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="6" t="n"/>
+      <c r="F42" s="6" t="n"/>
+      <c r="G42" s="6" t="n"/>
+      <c r="H42" s="6" t="n"/>
+      <c r="I42" s="6" t="n"/>
     </row>
     <row r="43" ht="26" customHeight="1"/>
     <row r="44" ht="26" customHeight="1">
@@ -2125,30 +2137,30 @@
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
-      <c r="G44" s="30" t="n"/>
-      <c r="H44" s="30" t="n"/>
-      <c r="I44" s="30" t="n"/>
-      <c r="K44" s="14" t="inlineStr">
+      <c r="G44" s="31" t="n"/>
+      <c r="H44" s="31" t="n"/>
+      <c r="I44" s="31" t="n"/>
+      <c r="K44" s="15" t="inlineStr">
         <is>
           <t>نام، سمت و امضای ارزیاب</t>
         </is>
       </c>
-      <c r="L44" s="14" t="n"/>
-      <c r="M44" s="14" t="n"/>
-      <c r="N44" s="14" t="n"/>
-      <c r="O44" s="14" t="n"/>
-      <c r="P44" s="14" t="n"/>
-      <c r="Q44" s="14" t="n"/>
-      <c r="R44" s="14" t="n"/>
-      <c r="S44" s="14" t="n"/>
-      <c r="U44" s="14" t="inlineStr">
+      <c r="L44" s="15" t="n"/>
+      <c r="M44" s="15" t="n"/>
+      <c r="N44" s="15" t="n"/>
+      <c r="O44" s="15" t="n"/>
+      <c r="P44" s="15" t="n"/>
+      <c r="Q44" s="15" t="n"/>
+      <c r="R44" s="15" t="n"/>
+      <c r="S44" s="15" t="n"/>
+      <c r="U44" s="15" t="inlineStr">
         <is>
           <t>تاریخ</t>
         </is>
       </c>
-      <c r="V44" s="14" t="n"/>
-      <c r="W44" s="14" t="n"/>
-      <c r="X44" s="14" t="n"/>
+      <c r="V44" s="15" t="n"/>
+      <c r="W44" s="15" t="n"/>
+      <c r="X44" s="15" t="n"/>
     </row>
     <row r="45" ht="26" customHeight="1">
       <c r="B45" s="2" t="n"/>
@@ -2156,22 +2168,22 @@
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="n"/>
       <c r="F45" s="2" t="n"/>
-      <c r="G45" s="30" t="n"/>
-      <c r="H45" s="30" t="n"/>
-      <c r="I45" s="30" t="n"/>
-      <c r="K45" s="31" t="n"/>
-      <c r="L45" s="31" t="n"/>
-      <c r="M45" s="31" t="n"/>
-      <c r="N45" s="31" t="n"/>
-      <c r="O45" s="31" t="n"/>
-      <c r="P45" s="31" t="n"/>
-      <c r="Q45" s="31" t="n"/>
-      <c r="R45" s="31" t="n"/>
-      <c r="S45" s="31" t="n"/>
-      <c r="U45" s="4" t="n"/>
-      <c r="V45" s="4" t="n"/>
-      <c r="W45" s="4" t="n"/>
-      <c r="X45" s="4" t="n"/>
+      <c r="G45" s="31" t="n"/>
+      <c r="H45" s="31" t="n"/>
+      <c r="I45" s="31" t="n"/>
+      <c r="K45" s="32" t="n"/>
+      <c r="L45" s="32" t="n"/>
+      <c r="M45" s="32" t="n"/>
+      <c r="N45" s="32" t="n"/>
+      <c r="O45" s="32" t="n"/>
+      <c r="P45" s="32" t="n"/>
+      <c r="Q45" s="32" t="n"/>
+      <c r="R45" s="32" t="n"/>
+      <c r="S45" s="32" t="n"/>
+      <c r="U45" s="5" t="n"/>
+      <c r="V45" s="5" t="n"/>
+      <c r="W45" s="5" t="n"/>
+      <c r="X45" s="5" t="n"/>
     </row>
     <row r="46" ht="26" customHeight="1">
       <c r="B46" s="2" t="n"/>
@@ -2179,22 +2191,22 @@
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="n"/>
-      <c r="G46" s="30" t="n"/>
-      <c r="H46" s="30" t="n"/>
-      <c r="I46" s="30" t="n"/>
-      <c r="K46" s="31" t="n"/>
-      <c r="L46" s="31" t="n"/>
-      <c r="M46" s="31" t="n"/>
-      <c r="N46" s="31" t="n"/>
-      <c r="O46" s="31" t="n"/>
-      <c r="P46" s="31" t="n"/>
-      <c r="Q46" s="31" t="n"/>
-      <c r="R46" s="31" t="n"/>
-      <c r="S46" s="31" t="n"/>
-      <c r="U46" s="4" t="n"/>
-      <c r="V46" s="4" t="n"/>
-      <c r="W46" s="4" t="n"/>
-      <c r="X46" s="4" t="n"/>
+      <c r="G46" s="31" t="n"/>
+      <c r="H46" s="31" t="n"/>
+      <c r="I46" s="31" t="n"/>
+      <c r="K46" s="32" t="n"/>
+      <c r="L46" s="32" t="n"/>
+      <c r="M46" s="32" t="n"/>
+      <c r="N46" s="32" t="n"/>
+      <c r="O46" s="32" t="n"/>
+      <c r="P46" s="32" t="n"/>
+      <c r="Q46" s="32" t="n"/>
+      <c r="R46" s="32" t="n"/>
+      <c r="S46" s="32" t="n"/>
+      <c r="U46" s="5" t="n"/>
+      <c r="V46" s="5" t="n"/>
+      <c r="W46" s="5" t="n"/>
+      <c r="X46" s="5" t="n"/>
     </row>
     <row r="47" ht="26" customHeight="1">
       <c r="B47" s="2" t="n"/>
@@ -2202,22 +2214,22 @@
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="n"/>
-      <c r="G47" s="30" t="n"/>
-      <c r="H47" s="30" t="n"/>
-      <c r="I47" s="30" t="n"/>
-      <c r="K47" s="31" t="n"/>
-      <c r="L47" s="31" t="n"/>
-      <c r="M47" s="31" t="n"/>
-      <c r="N47" s="31" t="n"/>
-      <c r="O47" s="31" t="n"/>
-      <c r="P47" s="31" t="n"/>
-      <c r="Q47" s="31" t="n"/>
-      <c r="R47" s="31" t="n"/>
-      <c r="S47" s="31" t="n"/>
-      <c r="U47" s="4" t="n"/>
-      <c r="V47" s="4" t="n"/>
-      <c r="W47" s="4" t="n"/>
-      <c r="X47" s="4" t="n"/>
+      <c r="G47" s="31" t="n"/>
+      <c r="H47" s="31" t="n"/>
+      <c r="I47" s="31" t="n"/>
+      <c r="K47" s="32" t="n"/>
+      <c r="L47" s="32" t="n"/>
+      <c r="M47" s="32" t="n"/>
+      <c r="N47" s="32" t="n"/>
+      <c r="O47" s="32" t="n"/>
+      <c r="P47" s="32" t="n"/>
+      <c r="Q47" s="32" t="n"/>
+      <c r="R47" s="32" t="n"/>
+      <c r="S47" s="32" t="n"/>
+      <c r="U47" s="5" t="n"/>
+      <c r="V47" s="5" t="n"/>
+      <c r="W47" s="5" t="n"/>
+      <c r="X47" s="5" t="n"/>
     </row>
     <row r="48" ht="26" customHeight="1">
       <c r="B48" s="2" t="n"/>
@@ -2225,79 +2237,84 @@
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
-      <c r="G48" s="30" t="n"/>
-      <c r="H48" s="30" t="n"/>
-      <c r="I48" s="30" t="n"/>
-      <c r="K48" s="31" t="n"/>
-      <c r="L48" s="31" t="n"/>
-      <c r="M48" s="31" t="n"/>
-      <c r="N48" s="31" t="n"/>
-      <c r="O48" s="31" t="n"/>
-      <c r="P48" s="31" t="n"/>
-      <c r="Q48" s="31" t="n"/>
-      <c r="R48" s="31" t="n"/>
-      <c r="S48" s="31" t="n"/>
-      <c r="U48" s="4" t="n"/>
-      <c r="V48" s="4" t="n"/>
-      <c r="W48" s="4" t="n"/>
-      <c r="X48" s="4" t="n"/>
+      <c r="G48" s="31" t="n"/>
+      <c r="H48" s="31" t="n"/>
+      <c r="I48" s="31" t="n"/>
+      <c r="K48" s="32" t="n"/>
+      <c r="L48" s="32" t="n"/>
+      <c r="M48" s="32" t="n"/>
+      <c r="N48" s="32" t="n"/>
+      <c r="O48" s="32" t="n"/>
+      <c r="P48" s="32" t="n"/>
+      <c r="Q48" s="32" t="n"/>
+      <c r="R48" s="32" t="n"/>
+      <c r="S48" s="32" t="n"/>
+      <c r="U48" s="5" t="n"/>
+      <c r="V48" s="5" t="n"/>
+      <c r="W48" s="5" t="n"/>
+      <c r="X48" s="5" t="n"/>
     </row>
     <row r="49" ht="26" customHeight="1"/>
   </sheetData>
-  <mergeCells count="133">
+  <mergeCells count="134">
+    <mergeCell ref="H10:K11"/>
     <mergeCell ref="B42:D42"/>
-    <mergeCell ref="E14:H15"/>
-    <mergeCell ref="N8:R9"/>
     <mergeCell ref="G32:I33"/>
     <mergeCell ref="C31:E31"/>
+    <mergeCell ref="Q14:T15"/>
+    <mergeCell ref="L12:L13"/>
     <mergeCell ref="U37:W37"/>
-    <mergeCell ref="N10:R11"/>
     <mergeCell ref="U23:X23"/>
+    <mergeCell ref="B4:M5"/>
     <mergeCell ref="G24:I24"/>
     <mergeCell ref="L25:N25"/>
-    <mergeCell ref="P19:R19"/>
-    <mergeCell ref="I10:J11"/>
-    <mergeCell ref="K4:X5"/>
-    <mergeCell ref="B12:D13"/>
+    <mergeCell ref="E8:G9"/>
     <mergeCell ref="G26:I26"/>
+    <mergeCell ref="N12:P13"/>
     <mergeCell ref="B20:X21"/>
     <mergeCell ref="U31:X33"/>
-    <mergeCell ref="B14:D15"/>
+    <mergeCell ref="E10:G11"/>
+    <mergeCell ref="H16:K17"/>
+    <mergeCell ref="S19:T19"/>
+    <mergeCell ref="H12:K13"/>
+    <mergeCell ref="N14:P15"/>
     <mergeCell ref="U28:V28"/>
-    <mergeCell ref="E16:H17"/>
     <mergeCell ref="E36:F36"/>
+    <mergeCell ref="H18:K19"/>
+    <mergeCell ref="Q16:T17"/>
     <mergeCell ref="K39:S40"/>
-    <mergeCell ref="B6:D7"/>
-    <mergeCell ref="E18:H19"/>
-    <mergeCell ref="N12:R13"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="H14:K15"/>
     <mergeCell ref="U36:W36"/>
-    <mergeCell ref="N14:R15"/>
+    <mergeCell ref="U7:X13"/>
     <mergeCell ref="C25:E25"/>
-    <mergeCell ref="J14:J19"/>
     <mergeCell ref="G28:I28"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="E42:I42"/>
-    <mergeCell ref="B4:J5"/>
-    <mergeCell ref="L26:N26"/>
+    <mergeCell ref="L10:M11"/>
+    <mergeCell ref="E12:G13"/>
+    <mergeCell ref="G40:H40"/>
     <mergeCell ref="G30:I30"/>
     <mergeCell ref="B1:X2"/>
     <mergeCell ref="P24:S24"/>
-    <mergeCell ref="K6:M7"/>
-    <mergeCell ref="S7:X13"/>
+    <mergeCell ref="U14:X14"/>
+    <mergeCell ref="L26:N26"/>
     <mergeCell ref="O32:O33"/>
     <mergeCell ref="E38:F38"/>
     <mergeCell ref="G38:H38"/>
+    <mergeCell ref="E14:G15"/>
     <mergeCell ref="P26:S26"/>
-    <mergeCell ref="E6:H7"/>
-    <mergeCell ref="P18:R18"/>
+    <mergeCell ref="N18:P19"/>
     <mergeCell ref="B23:I23"/>
     <mergeCell ref="E40:F40"/>
+    <mergeCell ref="U6:X6"/>
+    <mergeCell ref="Q6:T7"/>
     <mergeCell ref="P25:S25"/>
+    <mergeCell ref="B6:D19"/>
     <mergeCell ref="U38:W38"/>
     <mergeCell ref="L36:N36"/>
-    <mergeCell ref="J12:J13"/>
+    <mergeCell ref="N4:X5"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="L6:L7"/>
     <mergeCell ref="U24:V24"/>
     <mergeCell ref="U40:W40"/>
     <mergeCell ref="C24:E24"/>
@@ -2306,77 +2323,73 @@
     <mergeCell ref="L37:N37"/>
     <mergeCell ref="C26:E26"/>
     <mergeCell ref="B35:I35"/>
+    <mergeCell ref="N6:P7"/>
     <mergeCell ref="P37:S37"/>
+    <mergeCell ref="Q8:T9"/>
     <mergeCell ref="P30:S30"/>
+    <mergeCell ref="H6:K7"/>
     <mergeCell ref="E39:F39"/>
     <mergeCell ref="G39:H39"/>
-    <mergeCell ref="B16:D17"/>
+    <mergeCell ref="Q10:T11"/>
     <mergeCell ref="U44:X44"/>
+    <mergeCell ref="N16:P17"/>
     <mergeCell ref="K23:S23"/>
+    <mergeCell ref="M12:M13"/>
     <mergeCell ref="G37:H37"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="B18:D19"/>
     <mergeCell ref="U39:W39"/>
     <mergeCell ref="G29:I29"/>
-    <mergeCell ref="B8:D9"/>
     <mergeCell ref="C28:E28"/>
-    <mergeCell ref="S15:X19"/>
-    <mergeCell ref="I8:I9"/>
     <mergeCell ref="G31:I31"/>
     <mergeCell ref="L27:N27"/>
     <mergeCell ref="P32:S33"/>
     <mergeCell ref="G44:I48"/>
-    <mergeCell ref="N16:R17"/>
-    <mergeCell ref="N19:O19"/>
     <mergeCell ref="C30:E30"/>
-    <mergeCell ref="I14:I19"/>
     <mergeCell ref="P27:S27"/>
     <mergeCell ref="P36:S36"/>
     <mergeCell ref="E41:F41"/>
     <mergeCell ref="G41:H41"/>
-    <mergeCell ref="K8:M9"/>
+    <mergeCell ref="M14:M19"/>
     <mergeCell ref="U26:V26"/>
+    <mergeCell ref="E16:G17"/>
     <mergeCell ref="P28:S28"/>
-    <mergeCell ref="S14:X14"/>
-    <mergeCell ref="E8:H9"/>
-    <mergeCell ref="K10:M11"/>
     <mergeCell ref="U41:W41"/>
     <mergeCell ref="L30:N30"/>
     <mergeCell ref="K44:S44"/>
-    <mergeCell ref="J6:J7"/>
     <mergeCell ref="G36:H36"/>
+    <mergeCell ref="Q18:R18"/>
+    <mergeCell ref="E18:G19"/>
+    <mergeCell ref="S18:T18"/>
     <mergeCell ref="U27:V27"/>
-    <mergeCell ref="K16:M17"/>
-    <mergeCell ref="E10:H11"/>
     <mergeCell ref="L29:N29"/>
     <mergeCell ref="F32:F33"/>
     <mergeCell ref="U45:X48"/>
     <mergeCell ref="L38:N38"/>
-    <mergeCell ref="S6:X6"/>
     <mergeCell ref="C27:E27"/>
-    <mergeCell ref="K18:M19"/>
     <mergeCell ref="U35:X35"/>
-    <mergeCell ref="I12:I13"/>
+    <mergeCell ref="L8:L9"/>
     <mergeCell ref="U25:V25"/>
-    <mergeCell ref="N6:R7"/>
+    <mergeCell ref="M6:M7"/>
     <mergeCell ref="P29:S29"/>
+    <mergeCell ref="Q19:R19"/>
     <mergeCell ref="P38:S38"/>
     <mergeCell ref="K45:S48"/>
+    <mergeCell ref="L14:L19"/>
     <mergeCell ref="G25:I25"/>
     <mergeCell ref="P31:S31"/>
     <mergeCell ref="L31:N33"/>
     <mergeCell ref="U30:X30"/>
-    <mergeCell ref="K12:M13"/>
+    <mergeCell ref="U15:X19"/>
+    <mergeCell ref="N8:P9"/>
     <mergeCell ref="B44:F48"/>
+    <mergeCell ref="E6:G7"/>
     <mergeCell ref="B32:E33"/>
-    <mergeCell ref="B10:D11"/>
     <mergeCell ref="K31:K33"/>
+    <mergeCell ref="H8:K9"/>
+    <mergeCell ref="N10:P11"/>
     <mergeCell ref="U29:V29"/>
-    <mergeCell ref="E12:H13"/>
-    <mergeCell ref="K14:M15"/>
     <mergeCell ref="E37:F37"/>
     <mergeCell ref="C29:E29"/>
-    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="Q12:T13"/>
     <mergeCell ref="K35:S35"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
Photo as its own far-left section, banner spacing, fitted Excel columns
- Photo moved out of «اطلاعات فردی» into a separate section at the far
  left (beside «اطلاعات پرسنلی») in the form, view, print, Excel and Markdown
- «عملکردوتوانمندی کارکنان» banner separated from the tables above by an
  empty row; Excel page 2 starts with it
- Excel column widths fitted to measured content (+12 px); empty entry
  cells keep a minimum writing width by type

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Template/report_template.xlsx
+++ b/Template/report_template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="قالب" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'قالب'!$A$1:$Y$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'قالب'!$A$1:$AC$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -41,11 +41,6 @@
     </font>
     <font>
       <name val="B Nazanin"/>
-      <color rgb="009A9AB0"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="B Nazanin"/>
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="12"/>
@@ -64,6 +59,11 @@
       <name val="B Nazanin"/>
       <b val="1"/>
       <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="B Nazanin"/>
+      <color rgb="009A9AB0"/>
       <sz val="11"/>
     </font>
     <font>
@@ -240,33 +240,33 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" indent="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -275,7 +275,7 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -299,22 +299,22 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" indent="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -326,7 +326,7 @@
     <xf numFmtId="0" fontId="20" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:X48"/>
+  <dimension ref="B1:AB48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -722,6 +722,10 @@
     <col width="10" customWidth="1" min="23" max="23"/>
     <col width="10" customWidth="1" min="24" max="24"/>
     <col width="2" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="10" customWidth="1" min="28" max="28"/>
+    <col width="2" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -752,6 +756,10 @@
       <c r="V1" s="1" t="n"/>
       <c r="W1" s="1" t="n"/>
       <c r="X1" s="1" t="n"/>
+      <c r="Y1" s="1" t="n"/>
+      <c r="Z1" s="1" t="n"/>
+      <c r="AA1" s="1" t="n"/>
+      <c r="AB1" s="1" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="B2" s="1" t="n"/>
@@ -777,6 +785,10 @@
       <c r="V2" s="1" t="n"/>
       <c r="W2" s="1" t="n"/>
       <c r="X2" s="1" t="n"/>
+      <c r="Y2" s="1" t="n"/>
+      <c r="Z2" s="1" t="n"/>
+      <c r="AA2" s="1" t="n"/>
+      <c r="AB2" s="1" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1"/>
     <row r="4" ht="30" customHeight="1">
@@ -793,14 +805,14 @@
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>اطلاعات پرسنلی</t>
+        </is>
+      </c>
       <c r="L4" s="2" t="n"/>
       <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>اطلاعات پرسنلی</t>
-        </is>
-      </c>
+      <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="n"/>
       <c r="P4" s="2" t="n"/>
       <c r="Q4" s="2" t="n"/>
@@ -811,6 +823,13 @@
       <c r="V4" s="2" t="n"/>
       <c r="W4" s="2" t="n"/>
       <c r="X4" s="2" t="n"/>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
+          <t>عکس کارمند</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="n"/>
+      <c r="AB4" s="2" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="B5" s="2" t="n"/>
@@ -836,55 +855,61 @@
       <c r="V5" s="2" t="n"/>
       <c r="W5" s="2" t="n"/>
       <c r="X5" s="2" t="n"/>
+      <c r="Z5" s="2" t="n"/>
+      <c r="AA5" s="2" t="n"/>
+      <c r="AB5" s="2" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>عکس کارمند</t>
+          <t>نام ونام خانوادگی</t>
         </is>
       </c>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="3" t="n"/>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>نام ونام خانوادگی</t>
-        </is>
-      </c>
+      <c r="E6" s="4" t="n"/>
       <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>متأهل</t>
         </is>
       </c>
-      <c r="M6" s="6" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>مجرد</t>
         </is>
       </c>
-      <c r="N6" s="6" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>نوع استخدام</t>
         </is>
       </c>
-      <c r="O6" s="6" t="n"/>
-      <c r="P6" s="6" t="n"/>
-      <c r="Q6" s="5" t="n"/>
-      <c r="R6" s="5" t="n"/>
-      <c r="S6" s="5" t="n"/>
-      <c r="T6" s="5" t="n"/>
-      <c r="U6" s="7" t="inlineStr">
+      <c r="L6" s="5" t="n"/>
+      <c r="M6" s="5" t="n"/>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="4" t="n"/>
+      <c r="S6" s="6" t="inlineStr">
         <is>
           <t>سمت های قبلی:</t>
         </is>
       </c>
-      <c r="V6" s="7" t="n"/>
-      <c r="W6" s="7" t="n"/>
-      <c r="X6" s="7" t="n"/>
+      <c r="T6" s="6" t="n"/>
+      <c r="U6" s="6" t="n"/>
+      <c r="V6" s="6" t="n"/>
+      <c r="W6" s="6" t="n"/>
+      <c r="X6" s="6" t="n"/>
+      <c r="Z6" s="7" t="inlineStr">
+        <is>
+          <t>محل عکس</t>
+        </is>
+      </c>
+      <c r="AA6" s="7" t="n"/>
+      <c r="AB6" s="7" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="3" t="n"/>
@@ -893,64 +918,70 @@
       <c r="E7" s="4" t="n"/>
       <c r="F7" s="4" t="n"/>
       <c r="G7" s="4" t="n"/>
-      <c r="H7" s="5" t="n"/>
+      <c r="H7" s="4" t="n"/>
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="n"/>
-      <c r="L7" s="6" t="n"/>
-      <c r="M7" s="6" t="n"/>
-      <c r="N7" s="6" t="n"/>
-      <c r="O7" s="6" t="n"/>
-      <c r="P7" s="6" t="n"/>
-      <c r="Q7" s="5" t="n"/>
-      <c r="R7" s="5" t="n"/>
-      <c r="S7" s="5" t="n"/>
-      <c r="T7" s="5" t="n"/>
+      <c r="L7" s="5" t="n"/>
+      <c r="M7" s="5" t="n"/>
+      <c r="N7" s="4" t="n"/>
+      <c r="O7" s="4" t="n"/>
+      <c r="P7" s="4" t="n"/>
+      <c r="Q7" s="4" t="n"/>
+      <c r="R7" s="4" t="n"/>
+      <c r="S7" s="8" t="n"/>
+      <c r="T7" s="8" t="n"/>
       <c r="U7" s="8" t="n"/>
       <c r="V7" s="8" t="n"/>
       <c r="W7" s="8" t="n"/>
       <c r="X7" s="8" t="n"/>
+      <c r="Z7" s="7" t="n"/>
+      <c r="AA7" s="7" t="n"/>
+      <c r="AB7" s="7" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="B8" s="3" t="n"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>کدملی:</t>
+        </is>
+      </c>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="3" t="n"/>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>کدملی:</t>
-        </is>
-      </c>
+      <c r="E8" s="4" t="n"/>
       <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
-      <c r="L8" s="9" t="inlineStr">
+      <c r="H8" s="4" t="n"/>
+      <c r="I8" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="M8" s="9" t="inlineStr">
+      <c r="J8" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="N8" s="6" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>پست سازمانی</t>
         </is>
       </c>
-      <c r="O8" s="6" t="n"/>
-      <c r="P8" s="6" t="n"/>
-      <c r="Q8" s="5" t="n"/>
-      <c r="R8" s="5" t="n"/>
-      <c r="S8" s="5" t="n"/>
-      <c r="T8" s="5" t="n"/>
+      <c r="L8" s="5" t="n"/>
+      <c r="M8" s="5" t="n"/>
+      <c r="N8" s="4" t="n"/>
+      <c r="O8" s="4" t="n"/>
+      <c r="P8" s="4" t="n"/>
+      <c r="Q8" s="4" t="n"/>
+      <c r="R8" s="4" t="n"/>
+      <c r="S8" s="8" t="n"/>
+      <c r="T8" s="8" t="n"/>
       <c r="U8" s="8" t="n"/>
       <c r="V8" s="8" t="n"/>
       <c r="W8" s="8" t="n"/>
       <c r="X8" s="8" t="n"/>
+      <c r="Z8" s="7" t="n"/>
+      <c r="AA8" s="7" t="n"/>
+      <c r="AB8" s="7" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="B9" s="3" t="n"/>
@@ -959,60 +990,66 @@
       <c r="E9" s="4" t="n"/>
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="4" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
+      <c r="H9" s="4" t="n"/>
+      <c r="I9" s="9" t="n"/>
+      <c r="J9" s="9" t="n"/>
       <c r="K9" s="5" t="n"/>
-      <c r="L9" s="9" t="n"/>
-      <c r="M9" s="9" t="n"/>
-      <c r="N9" s="6" t="n"/>
-      <c r="O9" s="6" t="n"/>
-      <c r="P9" s="6" t="n"/>
-      <c r="Q9" s="5" t="n"/>
-      <c r="R9" s="5" t="n"/>
-      <c r="S9" s="5" t="n"/>
-      <c r="T9" s="5" t="n"/>
+      <c r="L9" s="5" t="n"/>
+      <c r="M9" s="5" t="n"/>
+      <c r="N9" s="4" t="n"/>
+      <c r="O9" s="4" t="n"/>
+      <c r="P9" s="4" t="n"/>
+      <c r="Q9" s="4" t="n"/>
+      <c r="R9" s="4" t="n"/>
+      <c r="S9" s="8" t="n"/>
+      <c r="T9" s="8" t="n"/>
       <c r="U9" s="8" t="n"/>
       <c r="V9" s="8" t="n"/>
       <c r="W9" s="8" t="n"/>
       <c r="X9" s="8" t="n"/>
+      <c r="Z9" s="7" t="n"/>
+      <c r="AA9" s="7" t="n"/>
+      <c r="AB9" s="7" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="B10" s="3" t="n"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>کدپرسنلی</t>
+        </is>
+      </c>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="3" t="n"/>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>کدپرسنلی</t>
-        </is>
-      </c>
+      <c r="E10" s="4" t="n"/>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>تعدادفرزندان</t>
+        </is>
+      </c>
       <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
-      <c r="L10" s="6" t="inlineStr">
-        <is>
-          <t>تعدادفرزندان</t>
-        </is>
-      </c>
-      <c r="M10" s="6" t="n"/>
-      <c r="N10" s="6" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>محل خدمت</t>
         </is>
       </c>
-      <c r="O10" s="6" t="n"/>
-      <c r="P10" s="6" t="n"/>
-      <c r="Q10" s="5" t="n"/>
-      <c r="R10" s="5" t="n"/>
-      <c r="S10" s="5" t="n"/>
-      <c r="T10" s="5" t="n"/>
+      <c r="L10" s="5" t="n"/>
+      <c r="M10" s="5" t="n"/>
+      <c r="N10" s="4" t="n"/>
+      <c r="O10" s="4" t="n"/>
+      <c r="P10" s="4" t="n"/>
+      <c r="Q10" s="4" t="n"/>
+      <c r="R10" s="4" t="n"/>
+      <c r="S10" s="8" t="n"/>
+      <c r="T10" s="8" t="n"/>
       <c r="U10" s="8" t="n"/>
       <c r="V10" s="8" t="n"/>
       <c r="W10" s="8" t="n"/>
       <c r="X10" s="8" t="n"/>
+      <c r="Z10" s="7" t="n"/>
+      <c r="AA10" s="7" t="n"/>
+      <c r="AB10" s="7" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="B11" s="3" t="n"/>
@@ -1021,64 +1058,70 @@
       <c r="E11" s="4" t="n"/>
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
-      <c r="H11" s="5" t="n"/>
+      <c r="H11" s="4" t="n"/>
       <c r="I11" s="5" t="n"/>
       <c r="J11" s="5" t="n"/>
       <c r="K11" s="5" t="n"/>
-      <c r="L11" s="6" t="n"/>
-      <c r="M11" s="6" t="n"/>
-      <c r="N11" s="6" t="n"/>
-      <c r="O11" s="6" t="n"/>
-      <c r="P11" s="6" t="n"/>
-      <c r="Q11" s="5" t="n"/>
-      <c r="R11" s="5" t="n"/>
-      <c r="S11" s="5" t="n"/>
-      <c r="T11" s="5" t="n"/>
+      <c r="L11" s="5" t="n"/>
+      <c r="M11" s="5" t="n"/>
+      <c r="N11" s="4" t="n"/>
+      <c r="O11" s="4" t="n"/>
+      <c r="P11" s="4" t="n"/>
+      <c r="Q11" s="4" t="n"/>
+      <c r="R11" s="4" t="n"/>
+      <c r="S11" s="8" t="n"/>
+      <c r="T11" s="8" t="n"/>
       <c r="U11" s="8" t="n"/>
       <c r="V11" s="8" t="n"/>
       <c r="W11" s="8" t="n"/>
       <c r="X11" s="8" t="n"/>
+      <c r="Z11" s="7" t="n"/>
+      <c r="AA11" s="7" t="n"/>
+      <c r="AB11" s="7" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>تاریخ تولد:</t>
+        </is>
+      </c>
       <c r="C12" s="3" t="n"/>
       <c r="D12" s="3" t="n"/>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>تاریخ تولد:</t>
-        </is>
-      </c>
+      <c r="E12" s="4" t="n"/>
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
-      <c r="K12" s="5" t="n"/>
-      <c r="L12" s="10" t="inlineStr">
+      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="10" t="inlineStr">
         <is>
           <t>دختر</t>
         </is>
       </c>
-      <c r="M12" s="11" t="inlineStr">
+      <c r="J12" s="11" t="inlineStr">
         <is>
           <t>پسر</t>
         </is>
       </c>
-      <c r="N12" s="6" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>تاریخ شروع به کار</t>
         </is>
       </c>
-      <c r="O12" s="6" t="n"/>
-      <c r="P12" s="6" t="n"/>
-      <c r="Q12" s="5" t="n"/>
-      <c r="R12" s="5" t="n"/>
-      <c r="S12" s="5" t="n"/>
-      <c r="T12" s="5" t="n"/>
+      <c r="L12" s="5" t="n"/>
+      <c r="M12" s="5" t="n"/>
+      <c r="N12" s="4" t="n"/>
+      <c r="O12" s="4" t="n"/>
+      <c r="P12" s="4" t="n"/>
+      <c r="Q12" s="4" t="n"/>
+      <c r="R12" s="4" t="n"/>
+      <c r="S12" s="8" t="n"/>
+      <c r="T12" s="8" t="n"/>
       <c r="U12" s="8" t="n"/>
       <c r="V12" s="8" t="n"/>
       <c r="W12" s="8" t="n"/>
       <c r="X12" s="8" t="n"/>
+      <c r="Z12" s="7" t="n"/>
+      <c r="AA12" s="7" t="n"/>
+      <c r="AB12" s="7" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="B13" s="3" t="n"/>
@@ -1087,60 +1130,66 @@
       <c r="E13" s="4" t="n"/>
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="4" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
+      <c r="H13" s="4" t="n"/>
+      <c r="I13" s="10" t="n"/>
+      <c r="J13" s="11" t="n"/>
       <c r="K13" s="5" t="n"/>
-      <c r="L13" s="10" t="n"/>
-      <c r="M13" s="11" t="n"/>
-      <c r="N13" s="6" t="n"/>
-      <c r="O13" s="6" t="n"/>
-      <c r="P13" s="6" t="n"/>
-      <c r="Q13" s="5" t="n"/>
-      <c r="R13" s="5" t="n"/>
-      <c r="S13" s="5" t="n"/>
-      <c r="T13" s="5" t="n"/>
+      <c r="L13" s="5" t="n"/>
+      <c r="M13" s="5" t="n"/>
+      <c r="N13" s="4" t="n"/>
+      <c r="O13" s="4" t="n"/>
+      <c r="P13" s="4" t="n"/>
+      <c r="Q13" s="4" t="n"/>
+      <c r="R13" s="4" t="n"/>
+      <c r="S13" s="8" t="n"/>
+      <c r="T13" s="8" t="n"/>
       <c r="U13" s="8" t="n"/>
       <c r="V13" s="8" t="n"/>
       <c r="W13" s="8" t="n"/>
       <c r="X13" s="8" t="n"/>
+      <c r="Z13" s="7" t="n"/>
+      <c r="AA13" s="7" t="n"/>
+      <c r="AB13" s="7" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>مدرک تحصیلی</t>
+        </is>
+      </c>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="3" t="n"/>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>مدرک تحصیلی</t>
-        </is>
-      </c>
+      <c r="E14" s="4" t="n"/>
       <c r="F14" s="4" t="n"/>
       <c r="G14" s="4" t="n"/>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="5" t="n"/>
-      <c r="K14" s="5" t="n"/>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>سوابق خدمتی/تجربی</t>
+        </is>
+      </c>
       <c r="L14" s="5" t="n"/>
       <c r="M14" s="5" t="n"/>
-      <c r="N14" s="6" t="inlineStr">
-        <is>
-          <t>سوابق خدمتی/تجربی</t>
-        </is>
-      </c>
-      <c r="O14" s="6" t="n"/>
-      <c r="P14" s="6" t="n"/>
-      <c r="Q14" s="5" t="n"/>
-      <c r="R14" s="5" t="n"/>
-      <c r="S14" s="5" t="n"/>
-      <c r="T14" s="5" t="n"/>
-      <c r="U14" s="7" t="inlineStr">
+      <c r="N14" s="4" t="n"/>
+      <c r="O14" s="4" t="n"/>
+      <c r="P14" s="4" t="n"/>
+      <c r="Q14" s="4" t="n"/>
+      <c r="R14" s="4" t="n"/>
+      <c r="S14" s="6" t="inlineStr">
         <is>
           <t>توقف پست:</t>
         </is>
       </c>
-      <c r="V14" s="7" t="n"/>
-      <c r="W14" s="7" t="n"/>
-      <c r="X14" s="7" t="n"/>
+      <c r="T14" s="6" t="n"/>
+      <c r="U14" s="6" t="n"/>
+      <c r="V14" s="6" t="n"/>
+      <c r="W14" s="6" t="n"/>
+      <c r="X14" s="6" t="n"/>
+      <c r="Z14" s="7" t="n"/>
+      <c r="AA14" s="7" t="n"/>
+      <c r="AB14" s="7" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="B15" s="3" t="n"/>
@@ -1149,56 +1198,62 @@
       <c r="E15" s="4" t="n"/>
       <c r="F15" s="4" t="n"/>
       <c r="G15" s="4" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
+      <c r="H15" s="4" t="n"/>
+      <c r="I15" s="4" t="n"/>
+      <c r="J15" s="4" t="n"/>
       <c r="K15" s="5" t="n"/>
       <c r="L15" s="5" t="n"/>
       <c r="M15" s="5" t="n"/>
-      <c r="N15" s="6" t="n"/>
-      <c r="O15" s="6" t="n"/>
-      <c r="P15" s="6" t="n"/>
-      <c r="Q15" s="5" t="n"/>
-      <c r="R15" s="5" t="n"/>
-      <c r="S15" s="5" t="n"/>
-      <c r="T15" s="5" t="n"/>
+      <c r="N15" s="4" t="n"/>
+      <c r="O15" s="4" t="n"/>
+      <c r="P15" s="4" t="n"/>
+      <c r="Q15" s="4" t="n"/>
+      <c r="R15" s="4" t="n"/>
+      <c r="S15" s="8" t="n"/>
+      <c r="T15" s="8" t="n"/>
       <c r="U15" s="8" t="n"/>
       <c r="V15" s="8" t="n"/>
       <c r="W15" s="8" t="n"/>
       <c r="X15" s="8" t="n"/>
+      <c r="Z15" s="7" t="n"/>
+      <c r="AA15" s="7" t="n"/>
+      <c r="AB15" s="7" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>رشته تحصیلی</t>
+        </is>
+      </c>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="n"/>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>رشته تحصیلی</t>
-        </is>
-      </c>
+      <c r="E16" s="4" t="n"/>
       <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
-      <c r="K16" s="5" t="n"/>
+      <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>سوابق آموزشی</t>
+        </is>
+      </c>
       <c r="L16" s="5" t="n"/>
       <c r="M16" s="5" t="n"/>
-      <c r="N16" s="6" t="inlineStr">
-        <is>
-          <t>سوابق آموزشی</t>
-        </is>
-      </c>
-      <c r="O16" s="6" t="n"/>
-      <c r="P16" s="6" t="n"/>
-      <c r="Q16" s="5" t="n"/>
-      <c r="R16" s="5" t="n"/>
-      <c r="S16" s="5" t="n"/>
-      <c r="T16" s="5" t="n"/>
+      <c r="N16" s="4" t="n"/>
+      <c r="O16" s="4" t="n"/>
+      <c r="P16" s="4" t="n"/>
+      <c r="Q16" s="4" t="n"/>
+      <c r="R16" s="4" t="n"/>
+      <c r="S16" s="8" t="n"/>
+      <c r="T16" s="8" t="n"/>
       <c r="U16" s="8" t="n"/>
       <c r="V16" s="8" t="n"/>
       <c r="W16" s="8" t="n"/>
       <c r="X16" s="8" t="n"/>
+      <c r="Z16" s="7" t="n"/>
+      <c r="AA16" s="7" t="n"/>
+      <c r="AB16" s="7" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="B17" s="3" t="n"/>
@@ -1207,64 +1262,70 @@
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="4" t="n"/>
       <c r="G17" s="4" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
+      <c r="H17" s="4" t="n"/>
+      <c r="I17" s="4" t="n"/>
+      <c r="J17" s="4" t="n"/>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="5" t="n"/>
       <c r="M17" s="5" t="n"/>
-      <c r="N17" s="6" t="n"/>
-      <c r="O17" s="6" t="n"/>
-      <c r="P17" s="6" t="n"/>
-      <c r="Q17" s="5" t="n"/>
-      <c r="R17" s="5" t="n"/>
-      <c r="S17" s="5" t="n"/>
-      <c r="T17" s="5" t="n"/>
+      <c r="N17" s="4" t="n"/>
+      <c r="O17" s="4" t="n"/>
+      <c r="P17" s="4" t="n"/>
+      <c r="Q17" s="4" t="n"/>
+      <c r="R17" s="4" t="n"/>
+      <c r="S17" s="8" t="n"/>
+      <c r="T17" s="8" t="n"/>
       <c r="U17" s="8" t="n"/>
       <c r="V17" s="8" t="n"/>
       <c r="W17" s="8" t="n"/>
       <c r="X17" s="8" t="n"/>
+      <c r="Z17" s="7" t="n"/>
+      <c r="AA17" s="7" t="n"/>
+      <c r="AB17" s="7" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="B18" s="3" t="n"/>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>شماره تماس:</t>
+        </is>
+      </c>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="3" t="n"/>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>شماره تماس:</t>
-        </is>
-      </c>
+      <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
-      <c r="H18" s="5" t="n"/>
-      <c r="I18" s="5" t="n"/>
-      <c r="J18" s="5" t="n"/>
-      <c r="K18" s="5" t="n"/>
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
+      <c r="J18" s="4" t="n"/>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>سوابق ارزیابی</t>
+        </is>
+      </c>
       <c r="L18" s="5" t="n"/>
       <c r="M18" s="5" t="n"/>
-      <c r="N18" s="6" t="inlineStr">
-        <is>
-          <t>سوابق ارزیابی</t>
-        </is>
-      </c>
-      <c r="O18" s="6" t="n"/>
-      <c r="P18" s="6" t="n"/>
-      <c r="Q18" s="12" t="inlineStr">
+      <c r="N18" s="12" t="inlineStr">
         <is>
           <t>تنبیهات</t>
         </is>
       </c>
+      <c r="O18" s="12" t="n"/>
+      <c r="P18" s="12" t="inlineStr">
+        <is>
+          <t>تشویق ها</t>
+        </is>
+      </c>
+      <c r="Q18" s="12" t="n"/>
       <c r="R18" s="12" t="n"/>
-      <c r="S18" s="12" t="inlineStr">
-        <is>
-          <t>تشویق ها</t>
-        </is>
-      </c>
-      <c r="T18" s="12" t="n"/>
+      <c r="S18" s="8" t="n"/>
+      <c r="T18" s="8" t="n"/>
       <c r="U18" s="8" t="n"/>
       <c r="V18" s="8" t="n"/>
       <c r="W18" s="8" t="n"/>
       <c r="X18" s="8" t="n"/>
+      <c r="Z18" s="7" t="n"/>
+      <c r="AA18" s="7" t="n"/>
+      <c r="AB18" s="7" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="B19" s="3" t="n"/>
@@ -1273,55 +1334,34 @@
       <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="n"/>
       <c r="G19" s="4" t="n"/>
-      <c r="H19" s="5" t="n"/>
-      <c r="I19" s="5" t="n"/>
-      <c r="J19" s="5" t="n"/>
+      <c r="H19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
+      <c r="J19" s="4" t="n"/>
       <c r="K19" s="5" t="n"/>
       <c r="L19" s="5" t="n"/>
       <c r="M19" s="5" t="n"/>
-      <c r="N19" s="6" t="n"/>
-      <c r="O19" s="6" t="n"/>
-      <c r="P19" s="6" t="n"/>
-      <c r="Q19" s="5" t="n"/>
-      <c r="R19" s="5" t="n"/>
-      <c r="S19" s="5" t="n"/>
-      <c r="T19" s="5" t="n"/>
+      <c r="N19" s="4" t="n"/>
+      <c r="O19" s="4" t="n"/>
+      <c r="P19" s="4" t="n"/>
+      <c r="Q19" s="4" t="n"/>
+      <c r="R19" s="4" t="n"/>
+      <c r="S19" s="8" t="n"/>
+      <c r="T19" s="8" t="n"/>
       <c r="U19" s="8" t="n"/>
       <c r="V19" s="8" t="n"/>
       <c r="W19" s="8" t="n"/>
       <c r="X19" s="8" t="n"/>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="B20" s="2" t="inlineStr">
+      <c r="Z19" s="7" t="n"/>
+      <c r="AA19" s="7" t="n"/>
+      <c r="AB19" s="7" t="n"/>
+    </row>
+    <row r="20" ht="14" customHeight="1"/>
+    <row r="21" ht="30" customHeight="1">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>عملکردوتوانمندی کارکنان</t>
         </is>
       </c>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n"/>
-      <c r="O20" s="2" t="n"/>
-      <c r="P20" s="2" t="n"/>
-      <c r="Q20" s="2" t="n"/>
-      <c r="R20" s="2" t="n"/>
-      <c r="S20" s="2" t="n"/>
-      <c r="T20" s="2" t="n"/>
-      <c r="U20" s="2" t="n"/>
-      <c r="V20" s="2" t="n"/>
-      <c r="W20" s="2" t="n"/>
-      <c r="X20" s="2" t="n"/>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="2" t="n"/>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="n"/>
@@ -1449,35 +1489,35 @@
       </c>
     </row>
     <row r="25" ht="26" customHeight="1">
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>۱</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>تخصص وتسلط بروظایف</t>
         </is>
       </c>
-      <c r="D25" s="5" t="n"/>
-      <c r="E25" s="5" t="n"/>
-      <c r="F25" s="5" t="n"/>
+      <c r="D25" s="4" t="n"/>
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4" t="n"/>
       <c r="G25" s="16" t="n"/>
       <c r="H25" s="16" t="n"/>
       <c r="I25" s="16" t="n"/>
-      <c r="K25" s="5" t="inlineStr">
+      <c r="K25" s="4" t="inlineStr">
         <is>
           <t>۱</t>
         </is>
       </c>
-      <c r="L25" s="5" t="inlineStr">
+      <c r="L25" s="4" t="inlineStr">
         <is>
           <t>ورود وخروج به موقع</t>
         </is>
       </c>
-      <c r="M25" s="5" t="n"/>
-      <c r="N25" s="5" t="n"/>
-      <c r="O25" s="5" t="n"/>
+      <c r="M25" s="4" t="n"/>
+      <c r="N25" s="4" t="n"/>
+      <c r="O25" s="4" t="n"/>
       <c r="P25" s="16" t="n"/>
       <c r="Q25" s="16" t="n"/>
       <c r="R25" s="16" t="n"/>
@@ -1500,35 +1540,35 @@
       </c>
     </row>
     <row r="26" ht="26" customHeight="1">
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>۲</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>دقت وکیفیت انجام کار</t>
         </is>
       </c>
-      <c r="D26" s="5" t="n"/>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="5" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
       <c r="G26" s="16" t="n"/>
       <c r="H26" s="16" t="n"/>
       <c r="I26" s="16" t="n"/>
-      <c r="K26" s="5" t="inlineStr">
+      <c r="K26" s="4" t="inlineStr">
         <is>
           <t>۲</t>
         </is>
       </c>
-      <c r="L26" s="5" t="inlineStr">
+      <c r="L26" s="4" t="inlineStr">
         <is>
           <t>میزان تأخیر/غیبت غیرموجه</t>
         </is>
       </c>
-      <c r="M26" s="5" t="n"/>
-      <c r="N26" s="5" t="n"/>
-      <c r="O26" s="5" t="n"/>
+      <c r="M26" s="4" t="n"/>
+      <c r="N26" s="4" t="n"/>
+      <c r="O26" s="4" t="n"/>
       <c r="P26" s="16" t="n"/>
       <c r="Q26" s="16" t="n"/>
       <c r="R26" s="16" t="n"/>
@@ -1551,35 +1591,35 @@
       </c>
     </row>
     <row r="27" ht="26" customHeight="1">
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>۳</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>مسئولیت پذیری</t>
         </is>
       </c>
-      <c r="D27" s="5" t="n"/>
-      <c r="E27" s="5" t="n"/>
-      <c r="F27" s="5" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
       <c r="G27" s="16" t="n"/>
       <c r="H27" s="16" t="n"/>
       <c r="I27" s="16" t="n"/>
-      <c r="K27" s="5" t="inlineStr">
+      <c r="K27" s="4" t="inlineStr">
         <is>
           <t>۳</t>
         </is>
       </c>
-      <c r="L27" s="5" t="inlineStr">
+      <c r="L27" s="4" t="inlineStr">
         <is>
           <t>رعایت شئونات اداری</t>
         </is>
       </c>
-      <c r="M27" s="5" t="n"/>
-      <c r="N27" s="5" t="n"/>
-      <c r="O27" s="5" t="n"/>
+      <c r="M27" s="4" t="n"/>
+      <c r="N27" s="4" t="n"/>
+      <c r="O27" s="4" t="n"/>
       <c r="P27" s="16" t="n"/>
       <c r="Q27" s="16" t="n"/>
       <c r="R27" s="16" t="n"/>
@@ -1602,35 +1642,35 @@
       </c>
     </row>
     <row r="28" ht="26" customHeight="1">
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>۴</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>توانائی حل مسئله ومدیریت امور</t>
         </is>
       </c>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="n"/>
       <c r="G28" s="16" t="n"/>
       <c r="H28" s="16" t="n"/>
       <c r="I28" s="16" t="n"/>
-      <c r="K28" s="5" t="inlineStr">
+      <c r="K28" s="4" t="inlineStr">
         <is>
           <t>۴</t>
         </is>
       </c>
-      <c r="L28" s="5" t="inlineStr">
+      <c r="L28" s="4" t="inlineStr">
         <is>
           <t>پایبندی به اصول اخلاق حرفه ای</t>
         </is>
       </c>
-      <c r="M28" s="5" t="n"/>
-      <c r="N28" s="5" t="n"/>
-      <c r="O28" s="5" t="n"/>
+      <c r="M28" s="4" t="n"/>
+      <c r="N28" s="4" t="n"/>
+      <c r="O28" s="4" t="n"/>
       <c r="P28" s="16" t="n"/>
       <c r="Q28" s="16" t="n"/>
       <c r="R28" s="16" t="n"/>
@@ -1653,35 +1693,35 @@
       </c>
     </row>
     <row r="29" ht="26" customHeight="1">
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>۵</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>همکاری وکارتیمی</t>
         </is>
       </c>
-      <c r="D29" s="5" t="n"/>
-      <c r="E29" s="5" t="n"/>
-      <c r="F29" s="5" t="n"/>
+      <c r="D29" s="4" t="n"/>
+      <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
       <c r="G29" s="16" t="n"/>
       <c r="H29" s="16" t="n"/>
       <c r="I29" s="16" t="n"/>
-      <c r="K29" s="5" t="inlineStr">
+      <c r="K29" s="4" t="inlineStr">
         <is>
           <t>۵</t>
         </is>
       </c>
-      <c r="L29" s="5" t="inlineStr">
+      <c r="L29" s="4" t="inlineStr">
         <is>
           <t>آراستگی وپوشش</t>
         </is>
       </c>
-      <c r="M29" s="5" t="n"/>
-      <c r="N29" s="5" t="n"/>
-      <c r="O29" s="5" t="n"/>
+      <c r="M29" s="4" t="n"/>
+      <c r="N29" s="4" t="n"/>
+      <c r="O29" s="4" t="n"/>
       <c r="P29" s="16" t="n"/>
       <c r="Q29" s="16" t="n"/>
       <c r="R29" s="16" t="n"/>
@@ -1704,77 +1744,77 @@
       </c>
     </row>
     <row r="30" ht="26" customHeight="1">
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>۶</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>تعامل وارتباط مؤثر</t>
         </is>
       </c>
-      <c r="D30" s="5" t="n"/>
-      <c r="E30" s="5" t="n"/>
-      <c r="F30" s="5" t="n"/>
+      <c r="D30" s="4" t="n"/>
+      <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="n"/>
       <c r="G30" s="16" t="n"/>
       <c r="H30" s="16" t="n"/>
       <c r="I30" s="16" t="n"/>
-      <c r="K30" s="5" t="inlineStr">
+      <c r="K30" s="4" t="inlineStr">
         <is>
           <t>۶</t>
         </is>
       </c>
-      <c r="L30" s="5" t="inlineStr">
+      <c r="L30" s="4" t="inlineStr">
         <is>
           <t>شرکت درمراسم مذهبی_فرهنگی</t>
         </is>
       </c>
-      <c r="M30" s="5" t="n"/>
-      <c r="N30" s="5" t="n"/>
-      <c r="O30" s="5" t="n"/>
+      <c r="M30" s="4" t="n"/>
+      <c r="N30" s="4" t="n"/>
+      <c r="O30" s="4" t="n"/>
       <c r="P30" s="16" t="n"/>
       <c r="Q30" s="16" t="n"/>
       <c r="R30" s="16" t="n"/>
       <c r="S30" s="16" t="n"/>
-      <c r="U30" s="4" t="inlineStr">
+      <c r="U30" s="3" t="inlineStr">
         <is>
           <t>توضیحات تکمیلی:</t>
         </is>
       </c>
-      <c r="V30" s="4" t="n"/>
-      <c r="W30" s="4" t="n"/>
-      <c r="X30" s="4" t="n"/>
+      <c r="V30" s="3" t="n"/>
+      <c r="W30" s="3" t="n"/>
+      <c r="X30" s="3" t="n"/>
     </row>
     <row r="31" ht="26" customHeight="1">
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>۷</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>ابتکاروارائه پیشنهادموثر</t>
         </is>
       </c>
-      <c r="D31" s="5" t="n"/>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n"/>
+      <c r="D31" s="4" t="n"/>
+      <c r="E31" s="4" t="n"/>
+      <c r="F31" s="4" t="n"/>
       <c r="G31" s="16" t="n"/>
       <c r="H31" s="16" t="n"/>
       <c r="I31" s="16" t="n"/>
-      <c r="K31" s="5" t="inlineStr">
+      <c r="K31" s="4" t="inlineStr">
         <is>
           <t>۷</t>
         </is>
       </c>
-      <c r="L31" s="5" t="inlineStr">
+      <c r="L31" s="4" t="inlineStr">
         <is>
           <t>تعهدات وتذکرات</t>
         </is>
       </c>
-      <c r="M31" s="5" t="n"/>
-      <c r="N31" s="5" t="n"/>
+      <c r="M31" s="4" t="n"/>
+      <c r="N31" s="4" t="n"/>
       <c r="O31" s="23" t="inlineStr">
         <is>
           <t>تذکر</t>
@@ -1798,14 +1838,14 @@
       <c r="C32" s="25" t="n"/>
       <c r="D32" s="25" t="n"/>
       <c r="E32" s="25" t="n"/>
-      <c r="F32" s="6" t="n"/>
+      <c r="F32" s="5" t="n"/>
       <c r="G32" s="26" t="n"/>
       <c r="H32" s="26" t="n"/>
       <c r="I32" s="26" t="n"/>
-      <c r="K32" s="5" t="n"/>
-      <c r="L32" s="5" t="n"/>
-      <c r="M32" s="5" t="n"/>
-      <c r="N32" s="5" t="n"/>
+      <c r="K32" s="4" t="n"/>
+      <c r="L32" s="4" t="n"/>
+      <c r="M32" s="4" t="n"/>
+      <c r="N32" s="4" t="n"/>
       <c r="O32" s="27" t="inlineStr">
         <is>
           <t>تعهد</t>
@@ -1825,14 +1865,14 @@
       <c r="C33" s="25" t="n"/>
       <c r="D33" s="25" t="n"/>
       <c r="E33" s="25" t="n"/>
-      <c r="F33" s="6" t="n"/>
+      <c r="F33" s="5" t="n"/>
       <c r="G33" s="26" t="n"/>
       <c r="H33" s="26" t="n"/>
       <c r="I33" s="26" t="n"/>
-      <c r="K33" s="5" t="n"/>
-      <c r="L33" s="5" t="n"/>
-      <c r="M33" s="5" t="n"/>
-      <c r="N33" s="5" t="n"/>
+      <c r="K33" s="4" t="n"/>
+      <c r="L33" s="4" t="n"/>
+      <c r="M33" s="4" t="n"/>
+      <c r="N33" s="4" t="n"/>
       <c r="O33" s="27" t="n"/>
       <c r="P33" s="16" t="n"/>
       <c r="Q33" s="16" t="n"/>
@@ -1947,31 +1987,31 @@
       <c r="X36" s="28" t="n"/>
     </row>
     <row r="37" ht="32" customHeight="1">
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>۱۴۰۰</t>
         </is>
       </c>
-      <c r="C37" s="5" t="n"/>
-      <c r="D37" s="5" t="n"/>
+      <c r="C37" s="4" t="n"/>
+      <c r="D37" s="4" t="n"/>
       <c r="E37" s="29" t="n"/>
       <c r="F37" s="29" t="n"/>
       <c r="G37" s="29" t="n"/>
       <c r="H37" s="29" t="n"/>
       <c r="I37" s="29" t="n"/>
-      <c r="K37" s="5" t="inlineStr">
+      <c r="K37" s="4" t="inlineStr">
         <is>
           <t>۱</t>
         </is>
       </c>
-      <c r="L37" s="5" t="inlineStr">
+      <c r="L37" s="4" t="inlineStr">
         <is>
           <t>رضایت مدیرمستقیم</t>
         </is>
       </c>
-      <c r="M37" s="5" t="n"/>
-      <c r="N37" s="5" t="n"/>
-      <c r="O37" s="5" t="n"/>
+      <c r="M37" s="4" t="n"/>
+      <c r="N37" s="4" t="n"/>
+      <c r="O37" s="4" t="n"/>
       <c r="P37" s="16" t="n"/>
       <c r="Q37" s="16" t="n"/>
       <c r="R37" s="16" t="n"/>
@@ -1986,31 +2026,31 @@
       <c r="X37" s="28" t="n"/>
     </row>
     <row r="38" ht="32" customHeight="1">
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>۱۴۰۱</t>
         </is>
       </c>
-      <c r="C38" s="5" t="n"/>
-      <c r="D38" s="5" t="n"/>
+      <c r="C38" s="4" t="n"/>
+      <c r="D38" s="4" t="n"/>
       <c r="E38" s="29" t="n"/>
       <c r="F38" s="29" t="n"/>
       <c r="G38" s="29" t="n"/>
       <c r="H38" s="29" t="n"/>
       <c r="I38" s="29" t="n"/>
-      <c r="K38" s="5" t="inlineStr">
+      <c r="K38" s="4" t="inlineStr">
         <is>
           <t>۲</t>
         </is>
       </c>
-      <c r="L38" s="5" t="inlineStr">
+      <c r="L38" s="4" t="inlineStr">
         <is>
           <t>رضایت ارباب رجوع</t>
         </is>
       </c>
-      <c r="M38" s="5" t="n"/>
-      <c r="N38" s="5" t="n"/>
-      <c r="O38" s="5" t="n"/>
+      <c r="M38" s="4" t="n"/>
+      <c r="N38" s="4" t="n"/>
+      <c r="O38" s="4" t="n"/>
       <c r="P38" s="16" t="n"/>
       <c r="Q38" s="16" t="n"/>
       <c r="R38" s="16" t="n"/>
@@ -2025,13 +2065,13 @@
       <c r="X38" s="28" t="n"/>
     </row>
     <row r="39" ht="32" customHeight="1">
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>۱۴۰۲</t>
         </is>
       </c>
-      <c r="C39" s="5" t="n"/>
-      <c r="D39" s="5" t="n"/>
+      <c r="C39" s="4" t="n"/>
+      <c r="D39" s="4" t="n"/>
       <c r="E39" s="29" t="n"/>
       <c r="F39" s="29" t="n"/>
       <c r="G39" s="29" t="n"/>
@@ -2060,13 +2100,13 @@
       <c r="X39" s="28" t="n"/>
     </row>
     <row r="40" ht="32" customHeight="1">
-      <c r="B40" s="6" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>۱۴۰۳</t>
         </is>
       </c>
-      <c r="C40" s="5" t="n"/>
-      <c r="D40" s="5" t="n"/>
+      <c r="C40" s="4" t="n"/>
+      <c r="D40" s="4" t="n"/>
       <c r="E40" s="29" t="n"/>
       <c r="F40" s="29" t="n"/>
       <c r="G40" s="29" t="n"/>
@@ -2091,13 +2131,13 @@
       <c r="X40" s="28" t="n"/>
     </row>
     <row r="41" ht="32" customHeight="1">
-      <c r="B41" s="6" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>۱۴۰۴</t>
         </is>
       </c>
-      <c r="C41" s="5" t="n"/>
-      <c r="D41" s="5" t="n"/>
+      <c r="C41" s="4" t="n"/>
+      <c r="D41" s="4" t="n"/>
       <c r="E41" s="29" t="n"/>
       <c r="F41" s="29" t="n"/>
       <c r="G41" s="29" t="n"/>
@@ -2120,11 +2160,11 @@
       </c>
       <c r="C42" s="15" t="n"/>
       <c r="D42" s="15" t="n"/>
-      <c r="E42" s="6" t="n"/>
-      <c r="F42" s="6" t="n"/>
-      <c r="G42" s="6" t="n"/>
-      <c r="H42" s="6" t="n"/>
-      <c r="I42" s="6" t="n"/>
+      <c r="E42" s="5" t="n"/>
+      <c r="F42" s="5" t="n"/>
+      <c r="G42" s="5" t="n"/>
+      <c r="H42" s="5" t="n"/>
+      <c r="I42" s="5" t="n"/>
     </row>
     <row r="43" ht="26" customHeight="1"/>
     <row r="44" ht="26" customHeight="1">
@@ -2180,10 +2220,10 @@
       <c r="Q45" s="32" t="n"/>
       <c r="R45" s="32" t="n"/>
       <c r="S45" s="32" t="n"/>
-      <c r="U45" s="5" t="n"/>
-      <c r="V45" s="5" t="n"/>
-      <c r="W45" s="5" t="n"/>
-      <c r="X45" s="5" t="n"/>
+      <c r="U45" s="4" t="n"/>
+      <c r="V45" s="4" t="n"/>
+      <c r="W45" s="4" t="n"/>
+      <c r="X45" s="4" t="n"/>
     </row>
     <row r="46" ht="26" customHeight="1">
       <c r="B46" s="2" t="n"/>
@@ -2203,10 +2243,10 @@
       <c r="Q46" s="32" t="n"/>
       <c r="R46" s="32" t="n"/>
       <c r="S46" s="32" t="n"/>
-      <c r="U46" s="5" t="n"/>
-      <c r="V46" s="5" t="n"/>
-      <c r="W46" s="5" t="n"/>
-      <c r="X46" s="5" t="n"/>
+      <c r="U46" s="4" t="n"/>
+      <c r="V46" s="4" t="n"/>
+      <c r="W46" s="4" t="n"/>
+      <c r="X46" s="4" t="n"/>
     </row>
     <row r="47" ht="26" customHeight="1">
       <c r="B47" s="2" t="n"/>
@@ -2226,10 +2266,10 @@
       <c r="Q47" s="32" t="n"/>
       <c r="R47" s="32" t="n"/>
       <c r="S47" s="32" t="n"/>
-      <c r="U47" s="5" t="n"/>
-      <c r="V47" s="5" t="n"/>
-      <c r="W47" s="5" t="n"/>
-      <c r="X47" s="5" t="n"/>
+      <c r="U47" s="4" t="n"/>
+      <c r="V47" s="4" t="n"/>
+      <c r="W47" s="4" t="n"/>
+      <c r="X47" s="4" t="n"/>
     </row>
     <row r="48" ht="26" customHeight="1">
       <c r="B48" s="2" t="n"/>
@@ -2249,154 +2289,155 @@
       <c r="Q48" s="32" t="n"/>
       <c r="R48" s="32" t="n"/>
       <c r="S48" s="32" t="n"/>
-      <c r="U48" s="5" t="n"/>
-      <c r="V48" s="5" t="n"/>
-      <c r="W48" s="5" t="n"/>
-      <c r="X48" s="5" t="n"/>
+      <c r="U48" s="4" t="n"/>
+      <c r="V48" s="4" t="n"/>
+      <c r="W48" s="4" t="n"/>
+      <c r="X48" s="4" t="n"/>
     </row>
     <row r="49" ht="26" customHeight="1"/>
   </sheetData>
-  <mergeCells count="134">
-    <mergeCell ref="H10:K11"/>
+  <mergeCells count="135">
     <mergeCell ref="B42:D42"/>
+    <mergeCell ref="E14:H15"/>
+    <mergeCell ref="N8:R9"/>
     <mergeCell ref="G32:I33"/>
     <mergeCell ref="C31:E31"/>
-    <mergeCell ref="Q14:T15"/>
-    <mergeCell ref="L12:L13"/>
     <mergeCell ref="U37:W37"/>
+    <mergeCell ref="N10:R11"/>
     <mergeCell ref="U23:X23"/>
-    <mergeCell ref="B4:M5"/>
     <mergeCell ref="G24:I24"/>
     <mergeCell ref="L25:N25"/>
-    <mergeCell ref="E8:G9"/>
+    <mergeCell ref="P19:R19"/>
+    <mergeCell ref="I10:J11"/>
+    <mergeCell ref="K4:X5"/>
+    <mergeCell ref="B12:D13"/>
     <mergeCell ref="G26:I26"/>
-    <mergeCell ref="N12:P13"/>
-    <mergeCell ref="B20:X21"/>
     <mergeCell ref="U31:X33"/>
-    <mergeCell ref="E10:G11"/>
-    <mergeCell ref="H16:K17"/>
-    <mergeCell ref="S19:T19"/>
-    <mergeCell ref="H12:K13"/>
-    <mergeCell ref="N14:P15"/>
+    <mergeCell ref="B14:D15"/>
+    <mergeCell ref="Z6:AB19"/>
     <mergeCell ref="U28:V28"/>
+    <mergeCell ref="E16:H17"/>
     <mergeCell ref="E36:F36"/>
-    <mergeCell ref="H18:K19"/>
-    <mergeCell ref="Q16:T17"/>
     <mergeCell ref="K39:S40"/>
-    <mergeCell ref="H14:K15"/>
+    <mergeCell ref="B6:D7"/>
+    <mergeCell ref="E18:H19"/>
+    <mergeCell ref="N12:R13"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="I6:I7"/>
     <mergeCell ref="U36:W36"/>
-    <mergeCell ref="U7:X13"/>
+    <mergeCell ref="N14:R15"/>
     <mergeCell ref="C25:E25"/>
+    <mergeCell ref="J14:J19"/>
     <mergeCell ref="G28:I28"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="E42:I42"/>
-    <mergeCell ref="L10:M11"/>
-    <mergeCell ref="E12:G13"/>
-    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="B4:J5"/>
     <mergeCell ref="G30:I30"/>
-    <mergeCell ref="B1:X2"/>
     <mergeCell ref="P24:S24"/>
-    <mergeCell ref="U14:X14"/>
     <mergeCell ref="L26:N26"/>
+    <mergeCell ref="K6:M7"/>
+    <mergeCell ref="S7:X13"/>
     <mergeCell ref="O32:O33"/>
     <mergeCell ref="E38:F38"/>
     <mergeCell ref="G38:H38"/>
-    <mergeCell ref="E14:G15"/>
     <mergeCell ref="P26:S26"/>
-    <mergeCell ref="N18:P19"/>
+    <mergeCell ref="E6:H7"/>
+    <mergeCell ref="P18:R18"/>
     <mergeCell ref="B23:I23"/>
     <mergeCell ref="E40:F40"/>
-    <mergeCell ref="U6:X6"/>
-    <mergeCell ref="Q6:T7"/>
     <mergeCell ref="P25:S25"/>
-    <mergeCell ref="B6:D19"/>
     <mergeCell ref="U38:W38"/>
     <mergeCell ref="L36:N36"/>
-    <mergeCell ref="N4:X5"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="J12:J13"/>
     <mergeCell ref="U24:V24"/>
     <mergeCell ref="U40:W40"/>
     <mergeCell ref="C24:E24"/>
     <mergeCell ref="G27:I27"/>
     <mergeCell ref="L28:N28"/>
     <mergeCell ref="L37:N37"/>
+    <mergeCell ref="B1:AB2"/>
     <mergeCell ref="C26:E26"/>
+    <mergeCell ref="Z4:AB5"/>
     <mergeCell ref="B35:I35"/>
-    <mergeCell ref="N6:P7"/>
     <mergeCell ref="P37:S37"/>
-    <mergeCell ref="Q8:T9"/>
     <mergeCell ref="P30:S30"/>
-    <mergeCell ref="H6:K7"/>
     <mergeCell ref="E39:F39"/>
     <mergeCell ref="G39:H39"/>
-    <mergeCell ref="Q10:T11"/>
+    <mergeCell ref="B16:D17"/>
     <mergeCell ref="U44:X44"/>
-    <mergeCell ref="N16:P17"/>
     <mergeCell ref="K23:S23"/>
-    <mergeCell ref="M12:M13"/>
     <mergeCell ref="G37:H37"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="B18:D19"/>
     <mergeCell ref="U39:W39"/>
     <mergeCell ref="G29:I29"/>
+    <mergeCell ref="B8:D9"/>
     <mergeCell ref="C28:E28"/>
+    <mergeCell ref="S15:X19"/>
+    <mergeCell ref="I8:I9"/>
     <mergeCell ref="G31:I31"/>
     <mergeCell ref="L27:N27"/>
     <mergeCell ref="P32:S33"/>
     <mergeCell ref="G44:I48"/>
+    <mergeCell ref="N16:R17"/>
+    <mergeCell ref="N19:O19"/>
     <mergeCell ref="C30:E30"/>
+    <mergeCell ref="I14:I19"/>
     <mergeCell ref="P27:S27"/>
     <mergeCell ref="P36:S36"/>
     <mergeCell ref="E41:F41"/>
     <mergeCell ref="G41:H41"/>
-    <mergeCell ref="M14:M19"/>
+    <mergeCell ref="K8:M9"/>
     <mergeCell ref="U26:V26"/>
-    <mergeCell ref="E16:G17"/>
     <mergeCell ref="P28:S28"/>
+    <mergeCell ref="S14:X14"/>
+    <mergeCell ref="E8:H9"/>
+    <mergeCell ref="K10:M11"/>
     <mergeCell ref="U41:W41"/>
     <mergeCell ref="L30:N30"/>
     <mergeCell ref="K44:S44"/>
+    <mergeCell ref="J6:J7"/>
     <mergeCell ref="G36:H36"/>
-    <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="E18:G19"/>
-    <mergeCell ref="S18:T18"/>
     <mergeCell ref="U27:V27"/>
+    <mergeCell ref="K16:M17"/>
+    <mergeCell ref="E10:H11"/>
     <mergeCell ref="L29:N29"/>
     <mergeCell ref="F32:F33"/>
     <mergeCell ref="U45:X48"/>
     <mergeCell ref="L38:N38"/>
+    <mergeCell ref="S6:X6"/>
     <mergeCell ref="C27:E27"/>
+    <mergeCell ref="K18:M19"/>
     <mergeCell ref="U35:X35"/>
-    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="I12:I13"/>
     <mergeCell ref="U25:V25"/>
-    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="B21:X21"/>
+    <mergeCell ref="N6:R7"/>
     <mergeCell ref="P29:S29"/>
-    <mergeCell ref="Q19:R19"/>
     <mergeCell ref="P38:S38"/>
     <mergeCell ref="K45:S48"/>
-    <mergeCell ref="L14:L19"/>
     <mergeCell ref="G25:I25"/>
     <mergeCell ref="P31:S31"/>
     <mergeCell ref="L31:N33"/>
     <mergeCell ref="U30:X30"/>
-    <mergeCell ref="U15:X19"/>
-    <mergeCell ref="N8:P9"/>
+    <mergeCell ref="K12:M13"/>
     <mergeCell ref="B44:F48"/>
-    <mergeCell ref="E6:G7"/>
     <mergeCell ref="B32:E33"/>
+    <mergeCell ref="B10:D11"/>
     <mergeCell ref="K31:K33"/>
-    <mergeCell ref="H8:K9"/>
-    <mergeCell ref="N10:P11"/>
     <mergeCell ref="U29:V29"/>
+    <mergeCell ref="E12:H13"/>
+    <mergeCell ref="K14:M15"/>
     <mergeCell ref="E37:F37"/>
     <mergeCell ref="C29:E29"/>
-    <mergeCell ref="Q12:T13"/>
+    <mergeCell ref="G40:H40"/>
     <mergeCell ref="K35:S35"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="21" min="0" max="16383" man="1"/>
+    <brk id="20" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Apply the user's Excel layout tuning
- Template column widths taken from the user's edited export
- Personal-info labels centred; colons removed from «کدملی» and «تاریخ تولد»
- Exports only widen a column when report data needs more room; fixed
  labels and entry room come from the tuned template widths

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Template/report_template.xlsx
+++ b/Template/report_template.xlsx
@@ -240,12 +240,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="2"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -298,6 +295,9 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -698,33 +698,33 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="5.5" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="8.5" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="10.83" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="6.5" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="2" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
-    <col width="10" customWidth="1" min="22" max="22"/>
-    <col width="10" customWidth="1" min="23" max="23"/>
-    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="11.5" customWidth="1" min="15" max="15"/>
+    <col width="6.5" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="3" customWidth="1" min="19" max="19"/>
+    <col width="10.83" customWidth="1" min="20" max="20"/>
+    <col width="10.5" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="3.5" customWidth="1" min="23" max="23"/>
+    <col width="6" customWidth="1" min="24" max="24"/>
     <col width="2" customWidth="1" min="25" max="25"/>
     <col width="10" customWidth="1" min="26" max="26"/>
-    <col width="10" customWidth="1" min="27" max="27"/>
-    <col width="10" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="13" customWidth="1" min="28" max="28"/>
     <col width="2" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
@@ -871,45 +871,45 @@
       <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="4" t="n"/>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>متأهل</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>مجرد</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>نوع استخدام</t>
         </is>
       </c>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="5" t="n"/>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="n"/>
       <c r="N6" s="4" t="n"/>
       <c r="O6" s="4" t="n"/>
       <c r="P6" s="4" t="n"/>
       <c r="Q6" s="4" t="n"/>
       <c r="R6" s="4" t="n"/>
-      <c r="S6" s="6" t="inlineStr">
+      <c r="S6" s="5" t="inlineStr">
         <is>
           <t>سمت های قبلی:</t>
         </is>
       </c>
-      <c r="T6" s="6" t="n"/>
-      <c r="U6" s="6" t="n"/>
-      <c r="V6" s="6" t="n"/>
-      <c r="W6" s="6" t="n"/>
-      <c r="X6" s="6" t="n"/>
-      <c r="Z6" s="7" t="inlineStr">
+      <c r="T6" s="5" t="n"/>
+      <c r="U6" s="5" t="n"/>
+      <c r="V6" s="5" t="n"/>
+      <c r="W6" s="5" t="n"/>
+      <c r="X6" s="5" t="n"/>
+      <c r="Z6" s="6" t="inlineStr">
         <is>
           <t>محل عکس</t>
         </is>
       </c>
-      <c r="AA6" s="7" t="n"/>
-      <c r="AB6" s="7" t="n"/>
+      <c r="AA6" s="6" t="n"/>
+      <c r="AB6" s="6" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="3" t="n"/>
@@ -919,30 +919,30 @@
       <c r="F7" s="4" t="n"/>
       <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="n"/>
       <c r="N7" s="4" t="n"/>
       <c r="O7" s="4" t="n"/>
       <c r="P7" s="4" t="n"/>
       <c r="Q7" s="4" t="n"/>
       <c r="R7" s="4" t="n"/>
-      <c r="S7" s="8" t="n"/>
-      <c r="T7" s="8" t="n"/>
-      <c r="U7" s="8" t="n"/>
-      <c r="V7" s="8" t="n"/>
-      <c r="W7" s="8" t="n"/>
-      <c r="X7" s="8" t="n"/>
-      <c r="Z7" s="7" t="n"/>
-      <c r="AA7" s="7" t="n"/>
-      <c r="AB7" s="7" t="n"/>
+      <c r="S7" s="7" t="n"/>
+      <c r="T7" s="7" t="n"/>
+      <c r="U7" s="7" t="n"/>
+      <c r="V7" s="7" t="n"/>
+      <c r="W7" s="7" t="n"/>
+      <c r="X7" s="7" t="n"/>
+      <c r="Z7" s="6" t="n"/>
+      <c r="AA7" s="6" t="n"/>
+      <c r="AB7" s="6" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>کدملی:</t>
+          <t>کدملی</t>
         </is>
       </c>
       <c r="C8" s="3" t="n"/>
@@ -951,37 +951,37 @@
       <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="n"/>
       <c r="H8" s="4" t="n"/>
-      <c r="I8" s="9" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="J8" s="9" t="inlineStr">
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>پست سازمانی</t>
         </is>
       </c>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="5" t="n"/>
+      <c r="L8" s="3" t="n"/>
+      <c r="M8" s="3" t="n"/>
       <c r="N8" s="4" t="n"/>
       <c r="O8" s="4" t="n"/>
       <c r="P8" s="4" t="n"/>
       <c r="Q8" s="4" t="n"/>
       <c r="R8" s="4" t="n"/>
-      <c r="S8" s="8" t="n"/>
-      <c r="T8" s="8" t="n"/>
-      <c r="U8" s="8" t="n"/>
-      <c r="V8" s="8" t="n"/>
-      <c r="W8" s="8" t="n"/>
-      <c r="X8" s="8" t="n"/>
-      <c r="Z8" s="7" t="n"/>
-      <c r="AA8" s="7" t="n"/>
-      <c r="AB8" s="7" t="n"/>
+      <c r="S8" s="7" t="n"/>
+      <c r="T8" s="7" t="n"/>
+      <c r="U8" s="7" t="n"/>
+      <c r="V8" s="7" t="n"/>
+      <c r="W8" s="7" t="n"/>
+      <c r="X8" s="7" t="n"/>
+      <c r="Z8" s="6" t="n"/>
+      <c r="AA8" s="6" t="n"/>
+      <c r="AB8" s="6" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="B9" s="3" t="n"/>
@@ -991,25 +991,25 @@
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="n"/>
-      <c r="I9" s="9" t="n"/>
-      <c r="J9" s="9" t="n"/>
-      <c r="K9" s="5" t="n"/>
-      <c r="L9" s="5" t="n"/>
-      <c r="M9" s="5" t="n"/>
+      <c r="I9" s="8" t="n"/>
+      <c r="J9" s="8" t="n"/>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n"/>
+      <c r="M9" s="3" t="n"/>
       <c r="N9" s="4" t="n"/>
       <c r="O9" s="4" t="n"/>
       <c r="P9" s="4" t="n"/>
       <c r="Q9" s="4" t="n"/>
       <c r="R9" s="4" t="n"/>
-      <c r="S9" s="8" t="n"/>
-      <c r="T9" s="8" t="n"/>
-      <c r="U9" s="8" t="n"/>
-      <c r="V9" s="8" t="n"/>
-      <c r="W9" s="8" t="n"/>
-      <c r="X9" s="8" t="n"/>
-      <c r="Z9" s="7" t="n"/>
-      <c r="AA9" s="7" t="n"/>
-      <c r="AB9" s="7" t="n"/>
+      <c r="S9" s="7" t="n"/>
+      <c r="T9" s="7" t="n"/>
+      <c r="U9" s="7" t="n"/>
+      <c r="V9" s="7" t="n"/>
+      <c r="W9" s="7" t="n"/>
+      <c r="X9" s="7" t="n"/>
+      <c r="Z9" s="6" t="n"/>
+      <c r="AA9" s="6" t="n"/>
+      <c r="AB9" s="6" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="B10" s="3" t="inlineStr">
@@ -1023,33 +1023,33 @@
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
       <c r="H10" s="4" t="n"/>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>تعدادفرزندان</t>
         </is>
       </c>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="inlineStr">
         <is>
           <t>محل خدمت</t>
         </is>
       </c>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
+      <c r="L10" s="3" t="n"/>
+      <c r="M10" s="3" t="n"/>
       <c r="N10" s="4" t="n"/>
       <c r="O10" s="4" t="n"/>
       <c r="P10" s="4" t="n"/>
       <c r="Q10" s="4" t="n"/>
       <c r="R10" s="4" t="n"/>
-      <c r="S10" s="8" t="n"/>
-      <c r="T10" s="8" t="n"/>
-      <c r="U10" s="8" t="n"/>
-      <c r="V10" s="8" t="n"/>
-      <c r="W10" s="8" t="n"/>
-      <c r="X10" s="8" t="n"/>
-      <c r="Z10" s="7" t="n"/>
-      <c r="AA10" s="7" t="n"/>
-      <c r="AB10" s="7" t="n"/>
+      <c r="S10" s="7" t="n"/>
+      <c r="T10" s="7" t="n"/>
+      <c r="U10" s="7" t="n"/>
+      <c r="V10" s="7" t="n"/>
+      <c r="W10" s="7" t="n"/>
+      <c r="X10" s="7" t="n"/>
+      <c r="Z10" s="6" t="n"/>
+      <c r="AA10" s="6" t="n"/>
+      <c r="AB10" s="6" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="B11" s="3" t="n"/>
@@ -1059,30 +1059,30 @@
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
-      <c r="L11" s="5" t="n"/>
-      <c r="M11" s="5" t="n"/>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="n"/>
+      <c r="M11" s="3" t="n"/>
       <c r="N11" s="4" t="n"/>
       <c r="O11" s="4" t="n"/>
       <c r="P11" s="4" t="n"/>
       <c r="Q11" s="4" t="n"/>
       <c r="R11" s="4" t="n"/>
-      <c r="S11" s="8" t="n"/>
-      <c r="T11" s="8" t="n"/>
-      <c r="U11" s="8" t="n"/>
-      <c r="V11" s="8" t="n"/>
-      <c r="W11" s="8" t="n"/>
-      <c r="X11" s="8" t="n"/>
-      <c r="Z11" s="7" t="n"/>
-      <c r="AA11" s="7" t="n"/>
-      <c r="AB11" s="7" t="n"/>
+      <c r="S11" s="7" t="n"/>
+      <c r="T11" s="7" t="n"/>
+      <c r="U11" s="7" t="n"/>
+      <c r="V11" s="7" t="n"/>
+      <c r="W11" s="7" t="n"/>
+      <c r="X11" s="7" t="n"/>
+      <c r="Z11" s="6" t="n"/>
+      <c r="AA11" s="6" t="n"/>
+      <c r="AB11" s="6" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>تاریخ تولد:</t>
+          <t>تاریخ تولد</t>
         </is>
       </c>
       <c r="C12" s="3" t="n"/>
@@ -1091,37 +1091,37 @@
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
       <c r="H12" s="4" t="n"/>
-      <c r="I12" s="10" t="inlineStr">
+      <c r="I12" s="9" t="inlineStr">
         <is>
           <t>دختر</t>
         </is>
       </c>
-      <c r="J12" s="11" t="inlineStr">
+      <c r="J12" s="10" t="inlineStr">
         <is>
           <t>پسر</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>تاریخ شروع به کار</t>
         </is>
       </c>
-      <c r="L12" s="5" t="n"/>
-      <c r="M12" s="5" t="n"/>
+      <c r="L12" s="3" t="n"/>
+      <c r="M12" s="3" t="n"/>
       <c r="N12" s="4" t="n"/>
       <c r="O12" s="4" t="n"/>
       <c r="P12" s="4" t="n"/>
       <c r="Q12" s="4" t="n"/>
       <c r="R12" s="4" t="n"/>
-      <c r="S12" s="8" t="n"/>
-      <c r="T12" s="8" t="n"/>
-      <c r="U12" s="8" t="n"/>
-      <c r="V12" s="8" t="n"/>
-      <c r="W12" s="8" t="n"/>
-      <c r="X12" s="8" t="n"/>
-      <c r="Z12" s="7" t="n"/>
-      <c r="AA12" s="7" t="n"/>
-      <c r="AB12" s="7" t="n"/>
+      <c r="S12" s="7" t="n"/>
+      <c r="T12" s="7" t="n"/>
+      <c r="U12" s="7" t="n"/>
+      <c r="V12" s="7" t="n"/>
+      <c r="W12" s="7" t="n"/>
+      <c r="X12" s="7" t="n"/>
+      <c r="Z12" s="6" t="n"/>
+      <c r="AA12" s="6" t="n"/>
+      <c r="AB12" s="6" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="B13" s="3" t="n"/>
@@ -1131,25 +1131,25 @@
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="n"/>
-      <c r="I13" s="10" t="n"/>
-      <c r="J13" s="11" t="n"/>
-      <c r="K13" s="5" t="n"/>
-      <c r="L13" s="5" t="n"/>
-      <c r="M13" s="5" t="n"/>
+      <c r="I13" s="9" t="n"/>
+      <c r="J13" s="10" t="n"/>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
+      <c r="M13" s="3" t="n"/>
       <c r="N13" s="4" t="n"/>
       <c r="O13" s="4" t="n"/>
       <c r="P13" s="4" t="n"/>
       <c r="Q13" s="4" t="n"/>
       <c r="R13" s="4" t="n"/>
-      <c r="S13" s="8" t="n"/>
-      <c r="T13" s="8" t="n"/>
-      <c r="U13" s="8" t="n"/>
-      <c r="V13" s="8" t="n"/>
-      <c r="W13" s="8" t="n"/>
-      <c r="X13" s="8" t="n"/>
-      <c r="Z13" s="7" t="n"/>
-      <c r="AA13" s="7" t="n"/>
-      <c r="AB13" s="7" t="n"/>
+      <c r="S13" s="7" t="n"/>
+      <c r="T13" s="7" t="n"/>
+      <c r="U13" s="7" t="n"/>
+      <c r="V13" s="7" t="n"/>
+      <c r="W13" s="7" t="n"/>
+      <c r="X13" s="7" t="n"/>
+      <c r="Z13" s="6" t="n"/>
+      <c r="AA13" s="6" t="n"/>
+      <c r="AB13" s="6" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="B14" s="3" t="inlineStr">
@@ -1165,31 +1165,31 @@
       <c r="H14" s="4" t="n"/>
       <c r="I14" s="4" t="n"/>
       <c r="J14" s="4" t="n"/>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K14" s="3" t="inlineStr">
         <is>
           <t>سوابق خدمتی/تجربی</t>
         </is>
       </c>
-      <c r="L14" s="5" t="n"/>
-      <c r="M14" s="5" t="n"/>
+      <c r="L14" s="3" t="n"/>
+      <c r="M14" s="3" t="n"/>
       <c r="N14" s="4" t="n"/>
       <c r="O14" s="4" t="n"/>
       <c r="P14" s="4" t="n"/>
       <c r="Q14" s="4" t="n"/>
       <c r="R14" s="4" t="n"/>
-      <c r="S14" s="6" t="inlineStr">
+      <c r="S14" s="5" t="inlineStr">
         <is>
           <t>توقف پست:</t>
         </is>
       </c>
-      <c r="T14" s="6" t="n"/>
-      <c r="U14" s="6" t="n"/>
-      <c r="V14" s="6" t="n"/>
-      <c r="W14" s="6" t="n"/>
-      <c r="X14" s="6" t="n"/>
-      <c r="Z14" s="7" t="n"/>
-      <c r="AA14" s="7" t="n"/>
-      <c r="AB14" s="7" t="n"/>
+      <c r="T14" s="5" t="n"/>
+      <c r="U14" s="5" t="n"/>
+      <c r="V14" s="5" t="n"/>
+      <c r="W14" s="5" t="n"/>
+      <c r="X14" s="5" t="n"/>
+      <c r="Z14" s="6" t="n"/>
+      <c r="AA14" s="6" t="n"/>
+      <c r="AB14" s="6" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="B15" s="3" t="n"/>
@@ -1201,23 +1201,23 @@
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="4" t="n"/>
       <c r="J15" s="4" t="n"/>
-      <c r="K15" s="5" t="n"/>
-      <c r="L15" s="5" t="n"/>
-      <c r="M15" s="5" t="n"/>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
+      <c r="M15" s="3" t="n"/>
       <c r="N15" s="4" t="n"/>
       <c r="O15" s="4" t="n"/>
       <c r="P15" s="4" t="n"/>
       <c r="Q15" s="4" t="n"/>
       <c r="R15" s="4" t="n"/>
-      <c r="S15" s="8" t="n"/>
-      <c r="T15" s="8" t="n"/>
-      <c r="U15" s="8" t="n"/>
-      <c r="V15" s="8" t="n"/>
-      <c r="W15" s="8" t="n"/>
-      <c r="X15" s="8" t="n"/>
-      <c r="Z15" s="7" t="n"/>
-      <c r="AA15" s="7" t="n"/>
-      <c r="AB15" s="7" t="n"/>
+      <c r="S15" s="7" t="n"/>
+      <c r="T15" s="7" t="n"/>
+      <c r="U15" s="7" t="n"/>
+      <c r="V15" s="7" t="n"/>
+      <c r="W15" s="7" t="n"/>
+      <c r="X15" s="7" t="n"/>
+      <c r="Z15" s="6" t="n"/>
+      <c r="AA15" s="6" t="n"/>
+      <c r="AB15" s="6" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="B16" s="3" t="inlineStr">
@@ -1233,27 +1233,27 @@
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="4" t="n"/>
       <c r="J16" s="4" t="n"/>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>سوابق آموزشی</t>
         </is>
       </c>
-      <c r="L16" s="5" t="n"/>
-      <c r="M16" s="5" t="n"/>
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="3" t="n"/>
       <c r="N16" s="4" t="n"/>
       <c r="O16" s="4" t="n"/>
       <c r="P16" s="4" t="n"/>
       <c r="Q16" s="4" t="n"/>
       <c r="R16" s="4" t="n"/>
-      <c r="S16" s="8" t="n"/>
-      <c r="T16" s="8" t="n"/>
-      <c r="U16" s="8" t="n"/>
-      <c r="V16" s="8" t="n"/>
-      <c r="W16" s="8" t="n"/>
-      <c r="X16" s="8" t="n"/>
-      <c r="Z16" s="7" t="n"/>
-      <c r="AA16" s="7" t="n"/>
-      <c r="AB16" s="7" t="n"/>
+      <c r="S16" s="7" t="n"/>
+      <c r="T16" s="7" t="n"/>
+      <c r="U16" s="7" t="n"/>
+      <c r="V16" s="7" t="n"/>
+      <c r="W16" s="7" t="n"/>
+      <c r="X16" s="7" t="n"/>
+      <c r="Z16" s="6" t="n"/>
+      <c r="AA16" s="6" t="n"/>
+      <c r="AB16" s="6" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="B17" s="3" t="n"/>
@@ -1265,23 +1265,23 @@
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="4" t="n"/>
       <c r="J17" s="4" t="n"/>
-      <c r="K17" s="5" t="n"/>
-      <c r="L17" s="5" t="n"/>
-      <c r="M17" s="5" t="n"/>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n"/>
+      <c r="M17" s="3" t="n"/>
       <c r="N17" s="4" t="n"/>
       <c r="O17" s="4" t="n"/>
       <c r="P17" s="4" t="n"/>
       <c r="Q17" s="4" t="n"/>
       <c r="R17" s="4" t="n"/>
-      <c r="S17" s="8" t="n"/>
-      <c r="T17" s="8" t="n"/>
-      <c r="U17" s="8" t="n"/>
-      <c r="V17" s="8" t="n"/>
-      <c r="W17" s="8" t="n"/>
-      <c r="X17" s="8" t="n"/>
-      <c r="Z17" s="7" t="n"/>
-      <c r="AA17" s="7" t="n"/>
-      <c r="AB17" s="7" t="n"/>
+      <c r="S17" s="7" t="n"/>
+      <c r="T17" s="7" t="n"/>
+      <c r="U17" s="7" t="n"/>
+      <c r="V17" s="7" t="n"/>
+      <c r="W17" s="7" t="n"/>
+      <c r="X17" s="7" t="n"/>
+      <c r="Z17" s="6" t="n"/>
+      <c r="AA17" s="6" t="n"/>
+      <c r="AB17" s="6" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="B18" s="3" t="inlineStr">
@@ -1297,35 +1297,35 @@
       <c r="H18" s="4" t="n"/>
       <c r="I18" s="4" t="n"/>
       <c r="J18" s="4" t="n"/>
-      <c r="K18" s="5" t="inlineStr">
+      <c r="K18" s="3" t="inlineStr">
         <is>
           <t>سوابق ارزیابی</t>
         </is>
       </c>
-      <c r="L18" s="5" t="n"/>
-      <c r="M18" s="5" t="n"/>
-      <c r="N18" s="12" t="inlineStr">
+      <c r="L18" s="3" t="n"/>
+      <c r="M18" s="3" t="n"/>
+      <c r="N18" s="11" t="inlineStr">
         <is>
           <t>تنبیهات</t>
         </is>
       </c>
-      <c r="O18" s="12" t="n"/>
-      <c r="P18" s="12" t="inlineStr">
+      <c r="O18" s="11" t="n"/>
+      <c r="P18" s="11" t="inlineStr">
         <is>
           <t>تشویق ها</t>
         </is>
       </c>
-      <c r="Q18" s="12" t="n"/>
-      <c r="R18" s="12" t="n"/>
-      <c r="S18" s="8" t="n"/>
-      <c r="T18" s="8" t="n"/>
-      <c r="U18" s="8" t="n"/>
-      <c r="V18" s="8" t="n"/>
-      <c r="W18" s="8" t="n"/>
-      <c r="X18" s="8" t="n"/>
-      <c r="Z18" s="7" t="n"/>
-      <c r="AA18" s="7" t="n"/>
-      <c r="AB18" s="7" t="n"/>
+      <c r="Q18" s="11" t="n"/>
+      <c r="R18" s="11" t="n"/>
+      <c r="S18" s="7" t="n"/>
+      <c r="T18" s="7" t="n"/>
+      <c r="U18" s="7" t="n"/>
+      <c r="V18" s="7" t="n"/>
+      <c r="W18" s="7" t="n"/>
+      <c r="X18" s="7" t="n"/>
+      <c r="Z18" s="6" t="n"/>
+      <c r="AA18" s="6" t="n"/>
+      <c r="AB18" s="6" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="B19" s="3" t="n"/>
@@ -1337,23 +1337,23 @@
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="4" t="n"/>
       <c r="J19" s="4" t="n"/>
-      <c r="K19" s="5" t="n"/>
-      <c r="L19" s="5" t="n"/>
-      <c r="M19" s="5" t="n"/>
+      <c r="K19" s="3" t="n"/>
+      <c r="L19" s="3" t="n"/>
+      <c r="M19" s="3" t="n"/>
       <c r="N19" s="4" t="n"/>
       <c r="O19" s="4" t="n"/>
       <c r="P19" s="4" t="n"/>
       <c r="Q19" s="4" t="n"/>
       <c r="R19" s="4" t="n"/>
-      <c r="S19" s="8" t="n"/>
-      <c r="T19" s="8" t="n"/>
-      <c r="U19" s="8" t="n"/>
-      <c r="V19" s="8" t="n"/>
-      <c r="W19" s="8" t="n"/>
-      <c r="X19" s="8" t="n"/>
-      <c r="Z19" s="7" t="n"/>
-      <c r="AA19" s="7" t="n"/>
-      <c r="AB19" s="7" t="n"/>
+      <c r="S19" s="7" t="n"/>
+      <c r="T19" s="7" t="n"/>
+      <c r="U19" s="7" t="n"/>
+      <c r="V19" s="7" t="n"/>
+      <c r="W19" s="7" t="n"/>
+      <c r="X19" s="7" t="n"/>
+      <c r="Z19" s="6" t="n"/>
+      <c r="AA19" s="6" t="n"/>
+      <c r="AB19" s="6" t="n"/>
     </row>
     <row r="20" ht="14" customHeight="1"/>
     <row r="21" ht="30" customHeight="1">
@@ -1387,102 +1387,102 @@
     </row>
     <row r="22" ht="26" customHeight="1"/>
     <row r="23" ht="26" customHeight="1">
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>ارزیابی توانمندی وشایستگی</t>
         </is>
       </c>
-      <c r="C23" s="13" t="n"/>
-      <c r="D23" s="13" t="n"/>
-      <c r="E23" s="13" t="n"/>
-      <c r="F23" s="13" t="n"/>
-      <c r="G23" s="13" t="n"/>
-      <c r="H23" s="13" t="n"/>
-      <c r="I23" s="13" t="n"/>
-      <c r="K23" s="13" t="inlineStr">
+      <c r="C23" s="12" t="n"/>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="12" t="n"/>
+      <c r="I23" s="12" t="n"/>
+      <c r="K23" s="12" t="inlineStr">
         <is>
           <t>کارنامه نظم وانضباط اداری</t>
         </is>
       </c>
-      <c r="L23" s="13" t="n"/>
-      <c r="M23" s="13" t="n"/>
-      <c r="N23" s="13" t="n"/>
-      <c r="O23" s="13" t="n"/>
-      <c r="P23" s="13" t="n"/>
-      <c r="Q23" s="13" t="n"/>
-      <c r="R23" s="13" t="n"/>
-      <c r="S23" s="13" t="n"/>
-      <c r="U23" s="14" t="inlineStr">
+      <c r="L23" s="12" t="n"/>
+      <c r="M23" s="12" t="n"/>
+      <c r="N23" s="12" t="n"/>
+      <c r="O23" s="12" t="n"/>
+      <c r="P23" s="12" t="n"/>
+      <c r="Q23" s="12" t="n"/>
+      <c r="R23" s="12" t="n"/>
+      <c r="S23" s="12" t="n"/>
+      <c r="U23" s="13" t="inlineStr">
         <is>
           <t>جمع بندی وپیشنهادات مدیریتی</t>
         </is>
       </c>
-      <c r="V23" s="14" t="n"/>
-      <c r="W23" s="14" t="n"/>
-      <c r="X23" s="14" t="n"/>
+      <c r="V23" s="13" t="n"/>
+      <c r="W23" s="13" t="n"/>
+      <c r="X23" s="13" t="n"/>
     </row>
     <row r="24" ht="26" customHeight="1">
-      <c r="B24" s="15" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>ردیف</t>
         </is>
       </c>
-      <c r="C24" s="15" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>شاخص</t>
         </is>
       </c>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="15" t="inlineStr">
+      <c r="D24" s="14" t="n"/>
+      <c r="E24" s="14" t="n"/>
+      <c r="F24" s="14" t="inlineStr">
         <is>
           <t>نمره</t>
         </is>
       </c>
-      <c r="G24" s="15" t="inlineStr">
+      <c r="G24" s="14" t="inlineStr">
         <is>
           <t>شرح</t>
         </is>
       </c>
-      <c r="H24" s="15" t="n"/>
-      <c r="I24" s="15" t="n"/>
-      <c r="K24" s="15" t="inlineStr">
+      <c r="H24" s="14" t="n"/>
+      <c r="I24" s="14" t="n"/>
+      <c r="K24" s="14" t="inlineStr">
         <is>
           <t>ردیف</t>
         </is>
       </c>
-      <c r="L24" s="15" t="inlineStr">
+      <c r="L24" s="14" t="inlineStr">
         <is>
           <t>شاخص</t>
         </is>
       </c>
-      <c r="M24" s="15" t="n"/>
-      <c r="N24" s="15" t="n"/>
-      <c r="O24" s="15" t="inlineStr">
+      <c r="M24" s="14" t="n"/>
+      <c r="N24" s="14" t="n"/>
+      <c r="O24" s="14" t="inlineStr">
         <is>
           <t>نمره</t>
         </is>
       </c>
-      <c r="P24" s="15" t="inlineStr">
+      <c r="P24" s="14" t="inlineStr">
         <is>
           <t>توضیحات/مستندات</t>
         </is>
       </c>
-      <c r="Q24" s="15" t="n"/>
-      <c r="R24" s="15" t="n"/>
-      <c r="S24" s="15" t="n"/>
-      <c r="U24" s="16" t="inlineStr">
+      <c r="Q24" s="14" t="n"/>
+      <c r="R24" s="14" t="n"/>
+      <c r="S24" s="14" t="n"/>
+      <c r="U24" s="15" t="inlineStr">
         <is>
           <t>شایسته تقدیروتشویق</t>
         </is>
       </c>
-      <c r="V24" s="16" t="n"/>
-      <c r="W24" s="17" t="inlineStr">
+      <c r="V24" s="15" t="n"/>
+      <c r="W24" s="16" t="inlineStr">
         <is>
           <t>✸</t>
         </is>
       </c>
-      <c r="X24" s="18" t="inlineStr">
+      <c r="X24" s="17" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
@@ -1502,9 +1502,9 @@
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
-      <c r="G25" s="16" t="n"/>
-      <c r="H25" s="16" t="n"/>
-      <c r="I25" s="16" t="n"/>
+      <c r="G25" s="15" t="n"/>
+      <c r="H25" s="15" t="n"/>
+      <c r="I25" s="15" t="n"/>
       <c r="K25" s="4" t="inlineStr">
         <is>
           <t>۱</t>
@@ -1518,22 +1518,22 @@
       <c r="M25" s="4" t="n"/>
       <c r="N25" s="4" t="n"/>
       <c r="O25" s="4" t="n"/>
-      <c r="P25" s="16" t="n"/>
-      <c r="Q25" s="16" t="n"/>
-      <c r="R25" s="16" t="n"/>
-      <c r="S25" s="16" t="n"/>
-      <c r="U25" s="16" t="inlineStr">
+      <c r="P25" s="15" t="n"/>
+      <c r="Q25" s="15" t="n"/>
+      <c r="R25" s="15" t="n"/>
+      <c r="S25" s="15" t="n"/>
+      <c r="U25" s="15" t="inlineStr">
         <is>
           <t>مناسب استمراردرمسئولیت فعلی</t>
         </is>
       </c>
-      <c r="V25" s="16" t="n"/>
-      <c r="W25" s="19" t="inlineStr">
+      <c r="V25" s="15" t="n"/>
+      <c r="W25" s="18" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="X25" s="18" t="inlineStr">
+      <c r="X25" s="17" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
@@ -1553,9 +1553,9 @@
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="4" t="n"/>
       <c r="F26" s="4" t="n"/>
-      <c r="G26" s="16" t="n"/>
-      <c r="H26" s="16" t="n"/>
-      <c r="I26" s="16" t="n"/>
+      <c r="G26" s="15" t="n"/>
+      <c r="H26" s="15" t="n"/>
+      <c r="I26" s="15" t="n"/>
       <c r="K26" s="4" t="inlineStr">
         <is>
           <t>۲</t>
@@ -1569,22 +1569,22 @@
       <c r="M26" s="4" t="n"/>
       <c r="N26" s="4" t="n"/>
       <c r="O26" s="4" t="n"/>
-      <c r="P26" s="16" t="n"/>
-      <c r="Q26" s="16" t="n"/>
-      <c r="R26" s="16" t="n"/>
-      <c r="S26" s="16" t="n"/>
-      <c r="U26" s="16" t="inlineStr">
+      <c r="P26" s="15" t="n"/>
+      <c r="Q26" s="15" t="n"/>
+      <c r="R26" s="15" t="n"/>
+      <c r="S26" s="15" t="n"/>
+      <c r="U26" s="15" t="inlineStr">
         <is>
           <t>شایسته ارتقای شغلی</t>
         </is>
       </c>
-      <c r="V26" s="16" t="n"/>
-      <c r="W26" s="20" t="inlineStr">
+      <c r="V26" s="15" t="n"/>
+      <c r="W26" s="19" t="inlineStr">
         <is>
           <t>⚑</t>
         </is>
       </c>
-      <c r="X26" s="18" t="inlineStr">
+      <c r="X26" s="17" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
@@ -1604,9 +1604,9 @@
       <c r="D27" s="4" t="n"/>
       <c r="E27" s="4" t="n"/>
       <c r="F27" s="4" t="n"/>
-      <c r="G27" s="16" t="n"/>
-      <c r="H27" s="16" t="n"/>
-      <c r="I27" s="16" t="n"/>
+      <c r="G27" s="15" t="n"/>
+      <c r="H27" s="15" t="n"/>
+      <c r="I27" s="15" t="n"/>
       <c r="K27" s="4" t="inlineStr">
         <is>
           <t>۳</t>
@@ -1620,22 +1620,22 @@
       <c r="M27" s="4" t="n"/>
       <c r="N27" s="4" t="n"/>
       <c r="O27" s="4" t="n"/>
-      <c r="P27" s="16" t="n"/>
-      <c r="Q27" s="16" t="n"/>
-      <c r="R27" s="16" t="n"/>
-      <c r="S27" s="16" t="n"/>
-      <c r="U27" s="16" t="inlineStr">
+      <c r="P27" s="15" t="n"/>
+      <c r="Q27" s="15" t="n"/>
+      <c r="R27" s="15" t="n"/>
+      <c r="S27" s="15" t="n"/>
+      <c r="U27" s="15" t="inlineStr">
         <is>
           <t>مستعدپذیرش مسئولیت بالاتر</t>
         </is>
       </c>
-      <c r="V27" s="16" t="n"/>
-      <c r="W27" s="21" t="inlineStr">
+      <c r="V27" s="15" t="n"/>
+      <c r="W27" s="20" t="inlineStr">
         <is>
           <t>☁</t>
         </is>
       </c>
-      <c r="X27" s="18" t="inlineStr">
+      <c r="X27" s="17" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
@@ -1655,9 +1655,9 @@
       <c r="D28" s="4" t="n"/>
       <c r="E28" s="4" t="n"/>
       <c r="F28" s="4" t="n"/>
-      <c r="G28" s="16" t="n"/>
-      <c r="H28" s="16" t="n"/>
-      <c r="I28" s="16" t="n"/>
+      <c r="G28" s="15" t="n"/>
+      <c r="H28" s="15" t="n"/>
+      <c r="I28" s="15" t="n"/>
       <c r="K28" s="4" t="inlineStr">
         <is>
           <t>۴</t>
@@ -1671,22 +1671,22 @@
       <c r="M28" s="4" t="n"/>
       <c r="N28" s="4" t="n"/>
       <c r="O28" s="4" t="n"/>
-      <c r="P28" s="16" t="n"/>
-      <c r="Q28" s="16" t="n"/>
-      <c r="R28" s="16" t="n"/>
-      <c r="S28" s="16" t="n"/>
-      <c r="U28" s="16" t="inlineStr">
+      <c r="P28" s="15" t="n"/>
+      <c r="Q28" s="15" t="n"/>
+      <c r="R28" s="15" t="n"/>
+      <c r="S28" s="15" t="n"/>
+      <c r="U28" s="15" t="inlineStr">
         <is>
           <t>نیازمندبرنامه بهبودعملکرد</t>
         </is>
       </c>
-      <c r="V28" s="16" t="n"/>
-      <c r="W28" s="22" t="inlineStr">
+      <c r="V28" s="15" t="n"/>
+      <c r="W28" s="21" t="inlineStr">
         <is>
           <t>■</t>
         </is>
       </c>
-      <c r="X28" s="18" t="inlineStr">
+      <c r="X28" s="17" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
@@ -1706,9 +1706,9 @@
       <c r="D29" s="4" t="n"/>
       <c r="E29" s="4" t="n"/>
       <c r="F29" s="4" t="n"/>
-      <c r="G29" s="16" t="n"/>
-      <c r="H29" s="16" t="n"/>
-      <c r="I29" s="16" t="n"/>
+      <c r="G29" s="15" t="n"/>
+      <c r="H29" s="15" t="n"/>
+      <c r="I29" s="15" t="n"/>
       <c r="K29" s="4" t="inlineStr">
         <is>
           <t>۵</t>
@@ -1722,22 +1722,22 @@
       <c r="M29" s="4" t="n"/>
       <c r="N29" s="4" t="n"/>
       <c r="O29" s="4" t="n"/>
-      <c r="P29" s="16" t="n"/>
-      <c r="Q29" s="16" t="n"/>
-      <c r="R29" s="16" t="n"/>
-      <c r="S29" s="16" t="n"/>
-      <c r="U29" s="16" t="inlineStr">
+      <c r="P29" s="15" t="n"/>
+      <c r="Q29" s="15" t="n"/>
+      <c r="R29" s="15" t="n"/>
+      <c r="S29" s="15" t="n"/>
+      <c r="U29" s="15" t="inlineStr">
         <is>
           <t>نیازمندبررسی مجددمسئولیت</t>
         </is>
       </c>
-      <c r="V29" s="16" t="n"/>
-      <c r="W29" s="22" t="inlineStr">
+      <c r="V29" s="15" t="n"/>
+      <c r="W29" s="21" t="inlineStr">
         <is>
           <t>■</t>
         </is>
       </c>
-      <c r="X29" s="18" t="inlineStr">
+      <c r="X29" s="17" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
@@ -1757,9 +1757,9 @@
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="n"/>
-      <c r="G30" s="16" t="n"/>
-      <c r="H30" s="16" t="n"/>
-      <c r="I30" s="16" t="n"/>
+      <c r="G30" s="15" t="n"/>
+      <c r="H30" s="15" t="n"/>
+      <c r="I30" s="15" t="n"/>
       <c r="K30" s="4" t="inlineStr">
         <is>
           <t>۶</t>
@@ -1773,18 +1773,18 @@
       <c r="M30" s="4" t="n"/>
       <c r="N30" s="4" t="n"/>
       <c r="O30" s="4" t="n"/>
-      <c r="P30" s="16" t="n"/>
-      <c r="Q30" s="16" t="n"/>
-      <c r="R30" s="16" t="n"/>
-      <c r="S30" s="16" t="n"/>
-      <c r="U30" s="3" t="inlineStr">
+      <c r="P30" s="15" t="n"/>
+      <c r="Q30" s="15" t="n"/>
+      <c r="R30" s="15" t="n"/>
+      <c r="S30" s="15" t="n"/>
+      <c r="U30" s="22" t="inlineStr">
         <is>
           <t>توضیحات تکمیلی:</t>
         </is>
       </c>
-      <c r="V30" s="3" t="n"/>
-      <c r="W30" s="3" t="n"/>
-      <c r="X30" s="3" t="n"/>
+      <c r="V30" s="22" t="n"/>
+      <c r="W30" s="22" t="n"/>
+      <c r="X30" s="22" t="n"/>
     </row>
     <row r="31" ht="26" customHeight="1">
       <c r="B31" s="4" t="inlineStr">
@@ -1800,9 +1800,9 @@
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="4" t="n"/>
       <c r="F31" s="4" t="n"/>
-      <c r="G31" s="16" t="n"/>
-      <c r="H31" s="16" t="n"/>
-      <c r="I31" s="16" t="n"/>
+      <c r="G31" s="15" t="n"/>
+      <c r="H31" s="15" t="n"/>
+      <c r="I31" s="15" t="n"/>
       <c r="K31" s="4" t="inlineStr">
         <is>
           <t>۷</t>
@@ -1820,10 +1820,10 @@
           <t>تذکر</t>
         </is>
       </c>
-      <c r="P31" s="16" t="n"/>
-      <c r="Q31" s="16" t="n"/>
-      <c r="R31" s="16" t="n"/>
-      <c r="S31" s="16" t="n"/>
+      <c r="P31" s="15" t="n"/>
+      <c r="Q31" s="15" t="n"/>
+      <c r="R31" s="15" t="n"/>
+      <c r="S31" s="15" t="n"/>
       <c r="U31" s="24" t="n"/>
       <c r="V31" s="24" t="n"/>
       <c r="W31" s="24" t="n"/>
@@ -1838,7 +1838,7 @@
       <c r="C32" s="25" t="n"/>
       <c r="D32" s="25" t="n"/>
       <c r="E32" s="25" t="n"/>
-      <c r="F32" s="5" t="n"/>
+      <c r="F32" s="3" t="n"/>
       <c r="G32" s="26" t="n"/>
       <c r="H32" s="26" t="n"/>
       <c r="I32" s="26" t="n"/>
@@ -1851,10 +1851,10 @@
           <t>تعهد</t>
         </is>
       </c>
-      <c r="P32" s="16" t="n"/>
-      <c r="Q32" s="16" t="n"/>
-      <c r="R32" s="16" t="n"/>
-      <c r="S32" s="16" t="n"/>
+      <c r="P32" s="15" t="n"/>
+      <c r="Q32" s="15" t="n"/>
+      <c r="R32" s="15" t="n"/>
+      <c r="S32" s="15" t="n"/>
       <c r="U32" s="24" t="n"/>
       <c r="V32" s="24" t="n"/>
       <c r="W32" s="24" t="n"/>
@@ -1865,7 +1865,7 @@
       <c r="C33" s="25" t="n"/>
       <c r="D33" s="25" t="n"/>
       <c r="E33" s="25" t="n"/>
-      <c r="F33" s="5" t="n"/>
+      <c r="F33" s="3" t="n"/>
       <c r="G33" s="26" t="n"/>
       <c r="H33" s="26" t="n"/>
       <c r="I33" s="26" t="n"/>
@@ -1874,10 +1874,10 @@
       <c r="M33" s="4" t="n"/>
       <c r="N33" s="4" t="n"/>
       <c r="O33" s="27" t="n"/>
-      <c r="P33" s="16" t="n"/>
-      <c r="Q33" s="16" t="n"/>
-      <c r="R33" s="16" t="n"/>
-      <c r="S33" s="16" t="n"/>
+      <c r="P33" s="15" t="n"/>
+      <c r="Q33" s="15" t="n"/>
+      <c r="R33" s="15" t="n"/>
+      <c r="S33" s="15" t="n"/>
       <c r="U33" s="24" t="n"/>
       <c r="V33" s="24" t="n"/>
       <c r="W33" s="24" t="n"/>
@@ -1885,109 +1885,109 @@
     </row>
     <row r="34" ht="26" customHeight="1"/>
     <row r="35" ht="26" customHeight="1">
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>سوابق ارزیابی ۵ سال گذشته</t>
         </is>
       </c>
-      <c r="C35" s="13" t="n"/>
-      <c r="D35" s="13" t="n"/>
-      <c r="E35" s="13" t="n"/>
-      <c r="F35" s="13" t="n"/>
-      <c r="G35" s="13" t="n"/>
-      <c r="H35" s="13" t="n"/>
-      <c r="I35" s="13" t="n"/>
-      <c r="K35" s="13" t="inlineStr">
+      <c r="C35" s="12" t="n"/>
+      <c r="D35" s="12" t="n"/>
+      <c r="E35" s="12" t="n"/>
+      <c r="F35" s="12" t="n"/>
+      <c r="G35" s="12" t="n"/>
+      <c r="H35" s="12" t="n"/>
+      <c r="I35" s="12" t="n"/>
+      <c r="K35" s="12" t="inlineStr">
         <is>
           <t>رضایت سنجی</t>
         </is>
       </c>
-      <c r="L35" s="13" t="n"/>
-      <c r="M35" s="13" t="n"/>
-      <c r="N35" s="13" t="n"/>
-      <c r="O35" s="13" t="n"/>
-      <c r="P35" s="13" t="n"/>
-      <c r="Q35" s="13" t="n"/>
-      <c r="R35" s="13" t="n"/>
-      <c r="S35" s="13" t="n"/>
-      <c r="U35" s="14" t="inlineStr">
+      <c r="L35" s="12" t="n"/>
+      <c r="M35" s="12" t="n"/>
+      <c r="N35" s="12" t="n"/>
+      <c r="O35" s="12" t="n"/>
+      <c r="P35" s="12" t="n"/>
+      <c r="Q35" s="12" t="n"/>
+      <c r="R35" s="12" t="n"/>
+      <c r="S35" s="12" t="n"/>
+      <c r="U35" s="13" t="inlineStr">
         <is>
           <t>جمع بندی نهائی ارزیابی عملکرد</t>
         </is>
       </c>
-      <c r="V35" s="14" t="n"/>
-      <c r="W35" s="14" t="n"/>
-      <c r="X35" s="14" t="n"/>
+      <c r="V35" s="13" t="n"/>
+      <c r="W35" s="13" t="n"/>
+      <c r="X35" s="13" t="n"/>
     </row>
     <row r="36" ht="26" customHeight="1">
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>سال</t>
         </is>
       </c>
-      <c r="C36" s="12" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>نمره کل</t>
         </is>
       </c>
-      <c r="D36" s="12" t="inlineStr">
+      <c r="D36" s="11" t="inlineStr">
         <is>
           <t>رتبه</t>
         </is>
       </c>
-      <c r="E36" s="12" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>روندعملکرد</t>
         </is>
       </c>
-      <c r="F36" s="12" t="n"/>
-      <c r="G36" s="12" t="inlineStr">
+      <c r="F36" s="11" t="n"/>
+      <c r="G36" s="11" t="inlineStr">
         <is>
           <t>نقاط قوت شاخص</t>
         </is>
       </c>
-      <c r="H36" s="12" t="n"/>
-      <c r="I36" s="12" t="inlineStr">
+      <c r="H36" s="11" t="n"/>
+      <c r="I36" s="11" t="inlineStr">
         <is>
           <t>مواردنیازمند بهبود</t>
         </is>
       </c>
-      <c r="K36" s="15" t="inlineStr">
+      <c r="K36" s="14" t="inlineStr">
         <is>
           <t>ردیف</t>
         </is>
       </c>
-      <c r="L36" s="15" t="inlineStr">
+      <c r="L36" s="14" t="inlineStr">
         <is>
           <t>شاخص</t>
         </is>
       </c>
-      <c r="M36" s="15" t="n"/>
-      <c r="N36" s="15" t="n"/>
-      <c r="O36" s="15" t="inlineStr">
+      <c r="M36" s="14" t="n"/>
+      <c r="N36" s="14" t="n"/>
+      <c r="O36" s="14" t="inlineStr">
         <is>
           <t>امتیاز</t>
         </is>
       </c>
-      <c r="P36" s="15" t="inlineStr">
+      <c r="P36" s="14" t="inlineStr">
         <is>
           <t>شرح</t>
         </is>
       </c>
-      <c r="Q36" s="15" t="n"/>
-      <c r="R36" s="15" t="n"/>
-      <c r="S36" s="15" t="n"/>
-      <c r="U36" s="16" t="inlineStr">
+      <c r="Q36" s="14" t="n"/>
+      <c r="R36" s="14" t="n"/>
+      <c r="S36" s="14" t="n"/>
+      <c r="U36" s="15" t="inlineStr">
         <is>
           <t>امتیازعملکردواحد/شعبه</t>
         </is>
       </c>
-      <c r="V36" s="16" t="n"/>
-      <c r="W36" s="16" t="n"/>
+      <c r="V36" s="15" t="n"/>
+      <c r="W36" s="15" t="n"/>
       <c r="X36" s="28" t="n"/>
     </row>
     <row r="37" ht="32" customHeight="1">
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>۱۴۰۰</t>
         </is>
@@ -2012,21 +2012,21 @@
       <c r="M37" s="4" t="n"/>
       <c r="N37" s="4" t="n"/>
       <c r="O37" s="4" t="n"/>
-      <c r="P37" s="16" t="n"/>
-      <c r="Q37" s="16" t="n"/>
-      <c r="R37" s="16" t="n"/>
-      <c r="S37" s="16" t="n"/>
-      <c r="U37" s="16" t="inlineStr">
+      <c r="P37" s="15" t="n"/>
+      <c r="Q37" s="15" t="n"/>
+      <c r="R37" s="15" t="n"/>
+      <c r="S37" s="15" t="n"/>
+      <c r="U37" s="15" t="inlineStr">
         <is>
           <t>امتیازعملکردفردی</t>
         </is>
       </c>
-      <c r="V37" s="16" t="n"/>
-      <c r="W37" s="16" t="n"/>
+      <c r="V37" s="15" t="n"/>
+      <c r="W37" s="15" t="n"/>
       <c r="X37" s="28" t="n"/>
     </row>
     <row r="38" ht="32" customHeight="1">
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>۱۴۰۱</t>
         </is>
@@ -2051,21 +2051,21 @@
       <c r="M38" s="4" t="n"/>
       <c r="N38" s="4" t="n"/>
       <c r="O38" s="4" t="n"/>
-      <c r="P38" s="16" t="n"/>
-      <c r="Q38" s="16" t="n"/>
-      <c r="R38" s="16" t="n"/>
-      <c r="S38" s="16" t="n"/>
-      <c r="U38" s="16" t="inlineStr">
+      <c r="P38" s="15" t="n"/>
+      <c r="Q38" s="15" t="n"/>
+      <c r="R38" s="15" t="n"/>
+      <c r="S38" s="15" t="n"/>
+      <c r="U38" s="15" t="inlineStr">
         <is>
           <t>امتیازتوانمندی حرفه ای</t>
         </is>
       </c>
-      <c r="V38" s="16" t="n"/>
-      <c r="W38" s="16" t="n"/>
+      <c r="V38" s="15" t="n"/>
+      <c r="W38" s="15" t="n"/>
       <c r="X38" s="28" t="n"/>
     </row>
     <row r="39" ht="32" customHeight="1">
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>۱۴۰۲</t>
         </is>
@@ -2090,17 +2090,17 @@
       <c r="Q39" s="30" t="n"/>
       <c r="R39" s="30" t="n"/>
       <c r="S39" s="30" t="n"/>
-      <c r="U39" s="16" t="inlineStr">
+      <c r="U39" s="15" t="inlineStr">
         <is>
           <t>امتیازنظم وانضباط اداری</t>
         </is>
       </c>
-      <c r="V39" s="16" t="n"/>
-      <c r="W39" s="16" t="n"/>
+      <c r="V39" s="15" t="n"/>
+      <c r="W39" s="15" t="n"/>
       <c r="X39" s="28" t="n"/>
     </row>
     <row r="40" ht="32" customHeight="1">
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>۱۴۰۳</t>
         </is>
@@ -2121,17 +2121,17 @@
       <c r="Q40" s="30" t="n"/>
       <c r="R40" s="30" t="n"/>
       <c r="S40" s="30" t="n"/>
-      <c r="U40" s="16" t="inlineStr">
+      <c r="U40" s="15" t="inlineStr">
         <is>
           <t>امتیازرضایت مدیر</t>
         </is>
       </c>
-      <c r="V40" s="16" t="n"/>
-      <c r="W40" s="16" t="n"/>
+      <c r="V40" s="15" t="n"/>
+      <c r="W40" s="15" t="n"/>
       <c r="X40" s="28" t="n"/>
     </row>
     <row r="41" ht="32" customHeight="1">
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>۱۴۰۴</t>
         </is>
@@ -2143,28 +2143,28 @@
       <c r="G41" s="29" t="n"/>
       <c r="H41" s="29" t="n"/>
       <c r="I41" s="29" t="n"/>
-      <c r="U41" s="16" t="inlineStr">
+      <c r="U41" s="15" t="inlineStr">
         <is>
           <t>امتیازتکریم ارباب رجوع</t>
         </is>
       </c>
-      <c r="V41" s="16" t="n"/>
-      <c r="W41" s="16" t="n"/>
+      <c r="V41" s="15" t="n"/>
+      <c r="W41" s="15" t="n"/>
       <c r="X41" s="28" t="n"/>
     </row>
     <row r="42" ht="26" customHeight="1">
-      <c r="B42" s="15" t="inlineStr">
+      <c r="B42" s="14" t="inlineStr">
         <is>
           <t>میانگین ۵ ساله</t>
         </is>
       </c>
-      <c r="C42" s="15" t="n"/>
-      <c r="D42" s="15" t="n"/>
-      <c r="E42" s="5" t="n"/>
-      <c r="F42" s="5" t="n"/>
-      <c r="G42" s="5" t="n"/>
-      <c r="H42" s="5" t="n"/>
-      <c r="I42" s="5" t="n"/>
+      <c r="C42" s="14" t="n"/>
+      <c r="D42" s="14" t="n"/>
+      <c r="E42" s="3" t="n"/>
+      <c r="F42" s="3" t="n"/>
+      <c r="G42" s="3" t="n"/>
+      <c r="H42" s="3" t="n"/>
+      <c r="I42" s="3" t="n"/>
     </row>
     <row r="43" ht="26" customHeight="1"/>
     <row r="44" ht="26" customHeight="1">
@@ -2180,27 +2180,27 @@
       <c r="G44" s="31" t="n"/>
       <c r="H44" s="31" t="n"/>
       <c r="I44" s="31" t="n"/>
-      <c r="K44" s="15" t="inlineStr">
+      <c r="K44" s="14" t="inlineStr">
         <is>
           <t>نام، سمت و امضای ارزیاب</t>
         </is>
       </c>
-      <c r="L44" s="15" t="n"/>
-      <c r="M44" s="15" t="n"/>
-      <c r="N44" s="15" t="n"/>
-      <c r="O44" s="15" t="n"/>
-      <c r="P44" s="15" t="n"/>
-      <c r="Q44" s="15" t="n"/>
-      <c r="R44" s="15" t="n"/>
-      <c r="S44" s="15" t="n"/>
-      <c r="U44" s="15" t="inlineStr">
+      <c r="L44" s="14" t="n"/>
+      <c r="M44" s="14" t="n"/>
+      <c r="N44" s="14" t="n"/>
+      <c r="O44" s="14" t="n"/>
+      <c r="P44" s="14" t="n"/>
+      <c r="Q44" s="14" t="n"/>
+      <c r="R44" s="14" t="n"/>
+      <c r="S44" s="14" t="n"/>
+      <c r="U44" s="14" t="inlineStr">
         <is>
           <t>تاریخ</t>
         </is>
       </c>
-      <c r="V44" s="15" t="n"/>
-      <c r="W44" s="15" t="n"/>
-      <c r="X44" s="15" t="n"/>
+      <c r="V44" s="14" t="n"/>
+      <c r="W44" s="14" t="n"/>
+      <c r="X44" s="14" t="n"/>
     </row>
     <row r="45" ht="26" customHeight="1">
       <c r="B45" s="2" t="n"/>

</xml_diff>